<commit_message>
Expand lexicon layers and fix relation resolution
Adds a large lexicon/data expansion (new dialect/register YAML layers, reference tables, and attribution/docs updates) and wires gender-scoped variants into lookup and display. Reworks core resolution with fixpoint-style normalization, identity-detour cancellation, exact-match pruning/grouping helpers, and multiple kinship-formatting fixes (including adoptive/step descendant naming and spouse-collateral depth handling). Introduces glyph-variant handling for 侄/姪, updates script conversion coverage, overhauls the UI workflow (removing language/origin mode controls, adding per-key variant menus, grouped “other names,” history restore, and layout/content policy changes), and adds extensive acceptance/verification coverage plus new validation scripts and release gating checks.
</commit_message>
<xml_diff>
--- a/Resource/Data/Reference/MumuyMainAccuracyCompact.xlsx
+++ b/Resource/Data/Reference/MumuyMainAccuracyCompact.xlsx
@@ -575,22 +575,22 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
+          <t>女兒 | 閨女|丫頭|妮子|囡囡|囡女|囡兒|乖囡|阿女|息女|女</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
           <t>女兒</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>女兒</t>
-        </is>
-      </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>女兒</t>
+          <t>女兒 | 閨女|丫頭|妮子|囡囡|囡女|囡兒|乖囡|阿女|息女|女</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -652,7 +652,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>外孫女</t>
+          <t>外孫女 | 外孫女兒|外孫囡</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -667,7 +667,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>外孫女</t>
+          <t>外孫女 | 外孫女兒|外孫囡</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -1114,7 +1114,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>外曾外孫婿</t>
+          <t>外曾外孫婿 | 外曾外孫女婿</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -1129,7 +1129,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>外曾外孫婿</t>
+          <t>外曾外孫婿 | 外曾外孫女婿</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1191,7 +1191,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>外曾外孫子</t>
+          <t>外曾外孫子 | 外曾外孫</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -1206,7 +1206,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>外曾外孫子</t>
+          <t>外曾外孫子 | 外曾外孫</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -1268,7 +1268,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>外玄孫女</t>
+          <t>外玄孫女 | 外元孫女</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>外玄孫女</t>
+          <t>外玄孫女 | 外元孫女</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -1345,7 +1345,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>外玄孫婿</t>
+          <t>外玄孫婿 | 外玄孫女婿</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -1360,7 +1360,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>外玄孫婿</t>
+          <t>外玄孫婿 | 外玄孫女婿</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -1422,7 +1422,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>外玄孫子</t>
+          <t>外玄孫子 | 外玄孫|外元孫</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -1437,7 +1437,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>外玄孫子</t>
+          <t>外玄孫子 | 外玄孫|外元孫</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -1499,7 +1499,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>外玄孫媳</t>
+          <t>外玄孫媳 | 外玄孫媳婦</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -1514,7 +1514,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>外玄孫媳</t>
+          <t>外玄孫媳 | 外玄孫媳婦</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -1576,7 +1576,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>外曾外孫媳</t>
+          <t>外曾外孫媳 | 外曾外孫媳婦</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -1591,7 +1591,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>外曾外孫媳</t>
+          <t>外曾外孫媳 | 外曾外孫媳婦</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
@@ -1653,7 +1653,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>外孫婿</t>
+          <t>外孫婿 | 外孫女婿</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
@@ -1668,7 +1668,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>外孫婿</t>
+          <t>外孫婿 | 外孫女婿</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -1730,7 +1730,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>外孫子 | 外孫</t>
+          <t>外孫子 | 外孫|外孫兒</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
@@ -1745,7 +1745,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>外孫子 | 外孫</t>
+          <t>外孫子 | 外孫|外孫兒</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
@@ -1807,7 +1807,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>外曾孫女</t>
+          <t>外曾孫女 | 重外孫女</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
@@ -1822,7 +1822,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>外曾孫女</t>
+          <t>外曾孫女 | 重外孫女</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
@@ -2192,7 +2192,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>外曾孫婿</t>
+          <t>外曾孫婿 | 外曾孫女婿|重外孫女婿</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
@@ -2207,7 +2207,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>外曾孫婿</t>
+          <t>外曾孫婿 | 外曾孫女婿|重外孫女婿</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
@@ -2269,7 +2269,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>外曾孫子</t>
+          <t>外曾孫子 | 重外孫|外曾孫</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
@@ -2284,7 +2284,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>外曾孫子</t>
+          <t>外曾孫子 | 重外孫|外曾孫</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
@@ -2346,7 +2346,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>外玄孫女</t>
+          <t>外玄孫女 | 外元孫女</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
@@ -2361,7 +2361,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>外玄孫女</t>
+          <t>外玄孫女 | 外元孫女</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
@@ -2423,7 +2423,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>外玄孫婿</t>
+          <t>外玄孫婿 | 外玄孫女婿</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
@@ -2438,7 +2438,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>外玄孫婿</t>
+          <t>外玄孫婿 | 外玄孫女婿</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
@@ -2500,7 +2500,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>外玄孫子</t>
+          <t>外玄孫子 | 外玄孫|外元孫</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
@@ -2515,7 +2515,7 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>外玄孫子</t>
+          <t>外玄孫子 | 外玄孫|外元孫</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
@@ -2577,7 +2577,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>外玄孫媳</t>
+          <t>外玄孫媳 | 外玄孫媳婦</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
@@ -2592,7 +2592,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>外玄孫媳</t>
+          <t>外玄孫媳 | 外玄孫媳婦</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
@@ -2654,7 +2654,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>外曾孫媳</t>
+          <t>外曾孫媳 | 外曾孫媳婦|外曾孫婦</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
@@ -2669,7 +2669,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>外曾孫媳</t>
+          <t>外曾孫媳 | 外曾孫媳婦|外曾孫婦</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
@@ -2731,7 +2731,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>外孫媳</t>
+          <t>外孫媳 | 外孫媳婦|外孫新婦|外孫婦</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
@@ -2746,7 +2746,7 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>外孫媳</t>
+          <t>外孫媳 | 外孫媳婦|外孫新婦|外孫婦</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
@@ -2808,7 +2808,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>女婿</t>
+          <t>女婿 | 姑爺|姑爺兒|女婿兒|囝婿|女婿子|囡婿|兒婿|子婿|息婿|小婿|快婿|郎婿|東床|半子|甥館|女夫</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
@@ -2823,7 +2823,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>女婿</t>
+          <t>女婿 | 姑爺|姑爺兒|女婿兒|囝婿|女婿子|囡婿|兒婿|子婿|息婿|小婿|快婿|郎婿|東床|半子|甥館|女夫</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
@@ -3116,7 +3116,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>姻姪</t>
+          <t>姻姪 | 世姪</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
@@ -3131,7 +3131,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>姻姪</t>
+          <t>姻姪 | 世姪</t>
         </is>
       </c>
       <c r="N36" t="inlineStr">
@@ -3732,7 +3732,7 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>姻姪</t>
+          <t>姻姪 | 世姪</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
@@ -3747,7 +3747,7 @@
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>姻姪</t>
+          <t>姻姪 | 世姪</t>
         </is>
       </c>
       <c r="N44" t="inlineStr">
@@ -4348,22 +4348,22 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
+          <t>父親 | 爸爸|老爸|老父親|爸|爹爹|爹|老爹|老爺子|阿爸|依爹|老漢|老漢兒|阿爹|老竇|爹地|阿父|父</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
           <t>父親</t>
         </is>
       </c>
-      <c r="J52" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="K52" t="inlineStr">
-        <is>
-          <t>父親</t>
-        </is>
-      </c>
       <c r="L52" t="inlineStr">
         <is>
-          <t>父親</t>
+          <t>父親 | 爸爸|老爸|老父親|爸|爹爹|爹|老爹|老爺子|阿爸|依爹|老漢|老漢兒|阿爹|老竇|爹地|阿父|父</t>
         </is>
       </c>
       <c r="N52" t="inlineStr">
@@ -4425,7 +4425,7 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>祖父 | 爺爺|阿公</t>
+          <t>祖父 | 爺爺|爺|阿公|祖公|阿爺|依爺|嗲嗲|亞爺|亞公|大父|祖翁</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
@@ -4440,7 +4440,7 @@
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t>祖父 | 爺爺|阿公</t>
+          <t>祖父 | 爺爺|爺|阿公|祖公|阿爺|依爺|嗲嗲|亞爺|亞公|大父|祖翁</t>
         </is>
       </c>
       <c r="N53" t="inlineStr">
@@ -4502,7 +4502,7 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>曾祖父 | 太爺爺|太公</t>
+          <t>曾祖父 | 太爺爺|太爺|老太爺|曾爺爺|太公|佬嗲|公太|曾祖|太翁</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
@@ -4517,7 +4517,7 @@
       </c>
       <c r="L54" t="inlineStr">
         <is>
-          <t>曾祖父 | 太爺爺|太公</t>
+          <t>曾祖父 | 太爺爺|太爺|老太爺|曾爺爺|太公|佬嗲|公太|曾祖|太翁</t>
         </is>
       </c>
       <c r="N54" t="inlineStr">
@@ -4579,7 +4579,7 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>高祖父</t>
+          <t>高祖父 | 祖太爺|祖太公|曾曾祖父</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
@@ -4594,7 +4594,7 @@
       </c>
       <c r="L55" t="inlineStr">
         <is>
-          <t>高祖父</t>
+          <t>高祖父 | 祖太爺|祖太公|曾曾祖父</t>
         </is>
       </c>
       <c r="N55" t="inlineStr">
@@ -7120,7 +7120,7 @@
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>高祖母</t>
+          <t>高祖母 | 祖太奶|祖太婆|曾曾祖母</t>
         </is>
       </c>
       <c r="J88" t="inlineStr">
@@ -7135,7 +7135,7 @@
       </c>
       <c r="L88" t="inlineStr">
         <is>
-          <t>高祖母</t>
+          <t>高祖母 | 祖太奶|祖太婆|曾曾祖母</t>
         </is>
       </c>
       <c r="N88" t="inlineStr">
@@ -7351,7 +7351,7 @@
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>從伯</t>
+          <t>從伯 | 從伯父|再從父</t>
         </is>
       </c>
       <c r="J91" t="inlineStr">
@@ -7366,7 +7366,7 @@
       </c>
       <c r="L91" t="inlineStr">
         <is>
-          <t>從伯</t>
+          <t>從伯 | 從伯父|再從父</t>
         </is>
       </c>
       <c r="N91" t="inlineStr">
@@ -7813,7 +7813,7 @@
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>從伯母</t>
+          <t>從伯母 | 再從母</t>
         </is>
       </c>
       <c r="J97" t="inlineStr">
@@ -7828,7 +7828,7 @@
       </c>
       <c r="L97" t="inlineStr">
         <is>
-          <t>從伯母</t>
+          <t>從伯母 | 再從母</t>
         </is>
       </c>
       <c r="N97" t="inlineStr">
@@ -8198,7 +8198,7 @@
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>從叔</t>
+          <t>從叔 | 從叔父|再從父</t>
         </is>
       </c>
       <c r="J102" t="inlineStr">
@@ -8213,7 +8213,7 @@
       </c>
       <c r="L102" t="inlineStr">
         <is>
-          <t>從叔</t>
+          <t>從叔 | 從叔父|再從父</t>
         </is>
       </c>
       <c r="N102" t="inlineStr">
@@ -8660,7 +8660,7 @@
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>從嬸</t>
+          <t>從嬸 | 再從母</t>
         </is>
       </c>
       <c r="J108" t="inlineStr">
@@ -8675,7 +8675,7 @@
       </c>
       <c r="L108" t="inlineStr">
         <is>
-          <t>從嬸</t>
+          <t>從嬸 | 再從母</t>
         </is>
       </c>
       <c r="N108" t="inlineStr">
@@ -8891,7 +8891,7 @@
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>曾祖母 | 太奶奶|太婆</t>
+          <t>曾祖母 | 太奶奶|太奶|老太奶|曾奶奶|太婆|太嬤|太姆|老娭毑|婆太</t>
         </is>
       </c>
       <c r="J111" t="inlineStr">
@@ -8906,7 +8906,7 @@
       </c>
       <c r="L111" t="inlineStr">
         <is>
-          <t>曾祖母 | 太奶奶|太婆</t>
+          <t>曾祖母 | 太奶奶|太奶|老太奶|曾奶奶|太婆|太嬤|太姆|老娭毑|婆太</t>
         </is>
       </c>
       <c r="N111" t="inlineStr">
@@ -9045,7 +9045,7 @@
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>高外祖母</t>
+          <t>高外祖母 | 高外婆</t>
         </is>
       </c>
       <c r="J113" t="inlineStr">
@@ -9060,7 +9060,7 @@
       </c>
       <c r="L113" t="inlineStr">
         <is>
-          <t>高外祖母</t>
+          <t>高外祖母 | 高外婆</t>
         </is>
       </c>
       <c r="N113" t="inlineStr">
@@ -9122,7 +9122,7 @@
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>伯祖父 | 大爺爺|伯公|大伯公</t>
+          <t>伯祖父 | 大爺爺|伯公|大伯公|大阿爺|大嗲|大公|伯祖|伯翁</t>
         </is>
       </c>
       <c r="J114" t="inlineStr">
@@ -9137,7 +9137,7 @@
       </c>
       <c r="L114" t="inlineStr">
         <is>
-          <t>伯祖父 | 大爺爺|伯公|大伯公</t>
+          <t>伯祖父 | 大爺爺|伯公|大伯公|大阿爺|大嗲|大公|伯祖|伯翁</t>
         </is>
       </c>
       <c r="N114" t="inlineStr">
@@ -9353,7 +9353,7 @@
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>堂伯</t>
+          <t>堂伯 | 從父</t>
         </is>
       </c>
       <c r="J117" t="inlineStr">
@@ -9368,7 +9368,7 @@
       </c>
       <c r="L117" t="inlineStr">
         <is>
-          <t>堂伯</t>
+          <t>堂伯 | 從父</t>
         </is>
       </c>
       <c r="N117" t="inlineStr">
@@ -9507,7 +9507,7 @@
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>從堂姪子</t>
+          <t>從堂姪子 | 從堂姪|三從子</t>
         </is>
       </c>
       <c r="J119" t="inlineStr">
@@ -9522,7 +9522,7 @@
       </c>
       <c r="L119" t="inlineStr">
         <is>
-          <t>從堂姪子</t>
+          <t>從堂姪子 | 從堂姪|三從子</t>
         </is>
       </c>
       <c r="N119" t="inlineStr">
@@ -9892,7 +9892,7 @@
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>伯祖母 | 大奶奶|伯奶奶|伯婆</t>
+          <t>伯祖母 | 大奶奶|伯奶奶|伯婆|姆婆|伯娭毑</t>
         </is>
       </c>
       <c r="J124" t="inlineStr">
@@ -9907,7 +9907,7 @@
       </c>
       <c r="L124" t="inlineStr">
         <is>
-          <t>伯祖母 | 大奶奶|伯奶奶|伯婆</t>
+          <t>伯祖母 | 大奶奶|伯奶奶|伯婆|姆婆|伯娭毑</t>
         </is>
       </c>
       <c r="N124" t="inlineStr">
@@ -9969,7 +9969,7 @@
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>姑祖母 | 姑奶奶|姑婆</t>
+          <t>姑祖母 | 姑奶奶|姑奶|姑婆|恩婆|姑娭毑|祖姑</t>
         </is>
       </c>
       <c r="J125" t="inlineStr">
@@ -9984,7 +9984,7 @@
       </c>
       <c r="L125" t="inlineStr">
         <is>
-          <t>姑祖母 | 姑奶奶|姑婆</t>
+          <t>姑祖母 | 姑奶奶|姑奶|姑婆|恩婆|姑娭毑|祖姑</t>
         </is>
       </c>
       <c r="N125" t="inlineStr">
@@ -10046,7 +10046,7 @@
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>姑祖父 | 姑爺爺|姑丈公|姑公</t>
+          <t>姑祖父 | 姑爺爺|姑丈公|姑公|恩爹|祖姑丈</t>
         </is>
       </c>
       <c r="J126" t="inlineStr">
@@ -10061,7 +10061,7 @@
       </c>
       <c r="L126" t="inlineStr">
         <is>
-          <t>姑祖父 | 姑爺爺|姑丈公|姑公</t>
+          <t>姑祖父 | 姑爺爺|姑丈公|姑公|恩爹|祖姑丈</t>
         </is>
       </c>
       <c r="N126" t="inlineStr">
@@ -10123,7 +10123,7 @@
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>叔祖父 | 小爺爺|叔公|小叔公</t>
+          <t>叔祖父 | 小爺爺|叔公|小叔公|幺爺|細嗲|叔祖|叔翁</t>
         </is>
       </c>
       <c r="J127" t="inlineStr">
@@ -10138,7 +10138,7 @@
       </c>
       <c r="L127" t="inlineStr">
         <is>
-          <t>叔祖父 | 小爺爺|叔公|小叔公</t>
+          <t>叔祖父 | 小爺爺|叔公|小叔公|幺爺|細嗲|叔祖|叔翁</t>
         </is>
       </c>
       <c r="N127" t="inlineStr">
@@ -10354,7 +10354,7 @@
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>堂叔</t>
+          <t>堂叔 | 從父</t>
         </is>
       </c>
       <c r="J130" t="inlineStr">
@@ -10369,7 +10369,7 @@
       </c>
       <c r="L130" t="inlineStr">
         <is>
-          <t>堂叔</t>
+          <t>堂叔 | 從父</t>
         </is>
       </c>
       <c r="N130" t="inlineStr">
@@ -10508,7 +10508,7 @@
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>從堂姪子</t>
+          <t>從堂姪子 | 從堂姪|三從子</t>
         </is>
       </c>
       <c r="J132" t="inlineStr">
@@ -10523,7 +10523,7 @@
       </c>
       <c r="L132" t="inlineStr">
         <is>
-          <t>從堂姪子</t>
+          <t>從堂姪子 | 從堂姪|三從子</t>
         </is>
       </c>
       <c r="N132" t="inlineStr">
@@ -10893,7 +10893,7 @@
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>叔祖母 | 叔婆|嬸婆</t>
+          <t>叔祖母 | 叔婆|嬸婆|幺奶|叔娭毑</t>
         </is>
       </c>
       <c r="J137" t="inlineStr">
@@ -10908,7 +10908,7 @@
       </c>
       <c r="L137" t="inlineStr">
         <is>
-          <t>叔祖母 | 叔婆|嬸婆</t>
+          <t>叔祖母 | 叔婆|嬸婆|幺奶|叔娭毑</t>
         </is>
       </c>
       <c r="N137" t="inlineStr">
@@ -10970,7 +10970,7 @@
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>姑祖母 | 姑奶奶|姑婆</t>
+          <t>姑祖母 | 姑奶奶|姑奶|姑婆|恩婆|姑娭毑|祖姑</t>
         </is>
       </c>
       <c r="J138" t="inlineStr">
@@ -10985,7 +10985,7 @@
       </c>
       <c r="L138" t="inlineStr">
         <is>
-          <t>姑祖母 | 姑奶奶|姑婆</t>
+          <t>姑祖母 | 姑奶奶|姑奶|姑婆|恩婆|姑娭毑|祖姑</t>
         </is>
       </c>
       <c r="N138" t="inlineStr">
@@ -11047,7 +11047,7 @@
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>姑祖父 | 姑爺爺|姑丈公|姑公</t>
+          <t>姑祖父 | 姑爺爺|姑丈公|姑公|恩爹|祖姑丈</t>
         </is>
       </c>
       <c r="J139" t="inlineStr">
@@ -11062,7 +11062,7 @@
       </c>
       <c r="L139" t="inlineStr">
         <is>
-          <t>姑祖父 | 姑爺爺|姑丈公|姑公</t>
+          <t>姑祖父 | 姑爺爺|姑丈公|姑公|恩爹|祖姑丈</t>
         </is>
       </c>
       <c r="N139" t="inlineStr">
@@ -11124,7 +11124,7 @@
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>祖母 | 奶奶|阿嬷</t>
+          <t>祖母 | 奶奶|奶|阿嬤|祖嫲|祖婆|依奶|阿奶|阿婆|親婆|娭毑|亞嬤|亞婆|嫲嫲|大母</t>
         </is>
       </c>
       <c r="J140" t="inlineStr">
@@ -11139,7 +11139,7 @@
       </c>
       <c r="L140" t="inlineStr">
         <is>
-          <t>祖母 | 奶奶|阿嬷</t>
+          <t>祖母 | 奶奶|奶|阿嬤|祖嫲|祖婆|依奶|阿奶|阿婆|親婆|娭毑|亞嬤|亞婆|嫲嫲|大母</t>
         </is>
       </c>
       <c r="N140" t="inlineStr">
@@ -11201,7 +11201,7 @@
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>曾外祖父</t>
+          <t>曾外祖父 | 太外爺|太外爺爺|太外公|曾外祖</t>
         </is>
       </c>
       <c r="J141" t="inlineStr">
@@ -11216,7 +11216,7 @@
       </c>
       <c r="L141" t="inlineStr">
         <is>
-          <t>曾外祖父</t>
+          <t>曾外祖父 | 太外爺|太外爺爺|太外公|曾外祖</t>
         </is>
       </c>
       <c r="N141" t="inlineStr">
@@ -11432,7 +11432,7 @@
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>曾外祖母</t>
+          <t>曾外祖母 | 太外奶|太外奶奶|太外婆</t>
         </is>
       </c>
       <c r="J144" t="inlineStr">
@@ -11447,7 +11447,7 @@
       </c>
       <c r="L144" t="inlineStr">
         <is>
-          <t>曾外祖母</t>
+          <t>曾外祖母 | 太外奶|太外奶奶|太外婆</t>
         </is>
       </c>
       <c r="N144" t="inlineStr">
@@ -11663,7 +11663,7 @@
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>舅祖父 | 舅爺|舅公</t>
+          <t>舅祖父 | 舅爺|舅爺爺|舅公|舅祖|太舅父</t>
         </is>
       </c>
       <c r="J147" t="inlineStr">
@@ -11678,7 +11678,7 @@
       </c>
       <c r="L147" t="inlineStr">
         <is>
-          <t>舅祖父 | 舅爺|舅公</t>
+          <t>舅祖父 | 舅爺|舅爺爺|舅公|舅祖|太舅父</t>
         </is>
       </c>
       <c r="N147" t="inlineStr">
@@ -11740,7 +11740,7 @@
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t>舅祖母 | 舅奶奶|舅婆</t>
+          <t>舅祖母 | 舅奶奶|妗婆|妗奶|舅婆|太舅母</t>
         </is>
       </c>
       <c r="J148" t="inlineStr">
@@ -11755,7 +11755,7 @@
       </c>
       <c r="L148" t="inlineStr">
         <is>
-          <t>舅祖母 | 舅奶奶|舅婆</t>
+          <t>舅祖母 | 舅奶奶|妗婆|妗奶|舅婆|太舅母</t>
         </is>
       </c>
       <c r="N148" t="inlineStr">
@@ -11817,7 +11817,7 @@
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>姨祖母 | 姨奶奶|姨婆</t>
+          <t>姨祖母 | 姨奶奶|姨奶|姨婆|姨娭毑</t>
         </is>
       </c>
       <c r="J149" t="inlineStr">
@@ -11832,7 +11832,7 @@
       </c>
       <c r="L149" t="inlineStr">
         <is>
-          <t>姨祖母 | 姨奶奶|姨婆</t>
+          <t>姨祖母 | 姨奶奶|姨奶|姨婆|姨娭毑</t>
         </is>
       </c>
       <c r="N149" t="inlineStr">
@@ -11894,7 +11894,7 @@
       </c>
       <c r="H150" t="inlineStr">
         <is>
-          <t>姨祖父 | 姨爺|姨公</t>
+          <t>姨祖父 | 姨爺|姨爺爺|姨公|姨公公|姨丈公</t>
         </is>
       </c>
       <c r="J150" t="inlineStr">
@@ -11909,7 +11909,7 @@
       </c>
       <c r="L150" t="inlineStr">
         <is>
-          <t>姨祖父 | 姨爺|姨公</t>
+          <t>姨祖父 | 姨爺|姨爺爺|姨公|姨公公|姨丈公</t>
         </is>
       </c>
       <c r="N150" t="inlineStr">
@@ -11971,7 +11971,7 @@
       </c>
       <c r="H151" t="inlineStr">
         <is>
-          <t>舅祖父 | 舅爺|舅公</t>
+          <t>舅祖父 | 舅爺|舅爺爺|舅公|舅祖|太舅父</t>
         </is>
       </c>
       <c r="J151" t="inlineStr">
@@ -11986,7 +11986,7 @@
       </c>
       <c r="L151" t="inlineStr">
         <is>
-          <t>舅祖父 | 舅爺|舅公</t>
+          <t>舅祖父 | 舅爺|舅爺爺|舅公|舅祖|太舅父</t>
         </is>
       </c>
       <c r="N151" t="inlineStr">
@@ -12048,7 +12048,7 @@
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>舅祖母 | 舅奶奶|舅婆</t>
+          <t>舅祖母 | 舅奶奶|妗婆|妗奶|舅婆|太舅母</t>
         </is>
       </c>
       <c r="J152" t="inlineStr">
@@ -12063,7 +12063,7 @@
       </c>
       <c r="L152" t="inlineStr">
         <is>
-          <t>舅祖母 | 舅奶奶|舅婆</t>
+          <t>舅祖母 | 舅奶奶|妗婆|妗奶|舅婆|太舅母</t>
         </is>
       </c>
       <c r="N152" t="inlineStr">
@@ -12125,7 +12125,7 @@
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>姨祖母 | 姨奶奶|姨婆</t>
+          <t>姨祖母 | 姨奶奶|姨奶|姨婆|姨娭毑</t>
         </is>
       </c>
       <c r="J153" t="inlineStr">
@@ -12140,7 +12140,7 @@
       </c>
       <c r="L153" t="inlineStr">
         <is>
-          <t>姨祖母 | 姨奶奶|姨婆</t>
+          <t>姨祖母 | 姨奶奶|姨奶|姨婆|姨娭毑</t>
         </is>
       </c>
       <c r="N153" t="inlineStr">
@@ -12202,7 +12202,7 @@
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t>姨祖父 | 姨爺|姨公</t>
+          <t>姨祖父 | 姨爺|姨爺爺|姨公|姨公公|姨丈公</t>
         </is>
       </c>
       <c r="J154" t="inlineStr">
@@ -12217,7 +12217,7 @@
       </c>
       <c r="L154" t="inlineStr">
         <is>
-          <t>姨祖父 | 姨爺|姨公</t>
+          <t>姨祖父 | 姨爺|姨爺爺|姨公|姨公公|姨丈公</t>
         </is>
       </c>
       <c r="N154" t="inlineStr">
@@ -12279,7 +12279,7 @@
       </c>
       <c r="H155" t="inlineStr">
         <is>
-          <t>伯父 | 伯伯</t>
+          <t>伯父 | 伯伯|大伯|伯|大爺|大大|阿伯|依伯|伯爸|大爹|大爸|大爸爸|伯爺|世父</t>
         </is>
       </c>
       <c r="J155" t="inlineStr">
@@ -12294,7 +12294,7 @@
       </c>
       <c r="L155" t="inlineStr">
         <is>
-          <t>伯父 | 伯伯</t>
+          <t>伯父 | 伯伯|大伯|伯|大爺|大大|阿伯|依伯|伯爸|大爹|大爸|大爸爸|伯爺|世父</t>
         </is>
       </c>
       <c r="N155" t="inlineStr">
@@ -12510,7 +12510,7 @@
       </c>
       <c r="H158" t="inlineStr">
         <is>
-          <t>堂外甥婿</t>
+          <t>堂外甥婿 | 堂外甥女婿</t>
         </is>
       </c>
       <c r="J158" t="inlineStr">
@@ -12525,7 +12525,7 @@
       </c>
       <c r="L158" t="inlineStr">
         <is>
-          <t>堂外甥婿</t>
+          <t>堂外甥婿 | 堂外甥女婿</t>
         </is>
       </c>
       <c r="N158" t="inlineStr">
@@ -12664,7 +12664,7 @@
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>堂外甥媳</t>
+          <t>堂外甥媳 | 堂外甥媳婦</t>
         </is>
       </c>
       <c r="J160" t="inlineStr">
@@ -12679,7 +12679,7 @@
       </c>
       <c r="L160" t="inlineStr">
         <is>
-          <t>堂外甥媳</t>
+          <t>堂外甥媳 | 堂外甥媳婦</t>
         </is>
       </c>
       <c r="N160" t="inlineStr">
@@ -12818,7 +12818,7 @@
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>堂兄</t>
+          <t>堂兄 | 堂哥</t>
         </is>
       </c>
       <c r="J162" t="inlineStr">
@@ -12833,7 +12833,7 @@
       </c>
       <c r="L162" t="inlineStr">
         <is>
-          <t>堂兄</t>
+          <t>堂兄 | 堂哥</t>
         </is>
       </c>
       <c r="N162" t="inlineStr">
@@ -12972,7 +12972,7 @@
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>堂姪婿</t>
+          <t>堂姪婿 | 堂姪女婿</t>
         </is>
       </c>
       <c r="J164" t="inlineStr">
@@ -12987,7 +12987,7 @@
       </c>
       <c r="L164" t="inlineStr">
         <is>
-          <t>堂姪婿</t>
+          <t>堂姪婿 | 堂姪女婿</t>
         </is>
       </c>
       <c r="N164" t="inlineStr">
@@ -13049,7 +13049,7 @@
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t>堂姪子</t>
+          <t>堂姪子 | 堂姪|再從子</t>
         </is>
       </c>
       <c r="J165" t="inlineStr">
@@ -13064,7 +13064,7 @@
       </c>
       <c r="L165" t="inlineStr">
         <is>
-          <t>堂姪子</t>
+          <t>堂姪子 | 堂姪|再從子</t>
         </is>
       </c>
       <c r="N165" t="inlineStr">
@@ -13126,7 +13126,7 @@
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>堂姪孫子</t>
+          <t>堂姪孫子 | 堂姪孫|再從孫</t>
         </is>
       </c>
       <c r="J166" t="inlineStr">
@@ -13141,7 +13141,7 @@
       </c>
       <c r="L166" t="inlineStr">
         <is>
-          <t>堂姪孫子</t>
+          <t>堂姪孫子 | 堂姪孫|再從孫</t>
         </is>
       </c>
       <c r="N166" t="inlineStr">
@@ -13357,7 +13357,7 @@
       </c>
       <c r="H169" t="inlineStr">
         <is>
-          <t>堂姪媳</t>
+          <t>堂姪媳 | 堂姪媳婦</t>
         </is>
       </c>
       <c r="J169" t="inlineStr">
@@ -13372,7 +13372,7 @@
       </c>
       <c r="L169" t="inlineStr">
         <is>
-          <t>堂姪媳</t>
+          <t>堂姪媳 | 堂姪媳婦</t>
         </is>
       </c>
       <c r="N169" t="inlineStr">
@@ -13434,7 +13434,7 @@
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>堂嫂</t>
+          <t>堂嫂 | 堂兄嫂</t>
         </is>
       </c>
       <c r="J170" t="inlineStr">
@@ -13449,7 +13449,7 @@
       </c>
       <c r="L170" t="inlineStr">
         <is>
-          <t>堂嫂</t>
+          <t>堂嫂 | 堂兄嫂</t>
         </is>
       </c>
       <c r="N170" t="inlineStr">
@@ -13511,7 +13511,7 @@
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>伯母</t>
+          <t>伯母 | 大娘|大媽|依姆|大嬤|姆|伯媽|伯娘|大媽媽|大姆媽|世母|伯婦</t>
         </is>
       </c>
       <c r="J171" t="inlineStr">
@@ -13526,7 +13526,7 @@
       </c>
       <c r="L171" t="inlineStr">
         <is>
-          <t>伯母</t>
+          <t>伯母 | 大娘|大媽|依姆|大嬤|姆|伯媽|伯娘|大媽媽|大姆媽|世母|伯婦</t>
         </is>
       </c>
       <c r="N171" t="inlineStr">
@@ -13588,7 +13588,7 @@
       </c>
       <c r="H172" t="inlineStr">
         <is>
-          <t>姑母 | 姑姑|姑媽</t>
+          <t>姑母 | 姑姑|大姑|姑|小姑|老姑|姑媽|姑嬤|姑仔|尕娘|嬢嬢|娘娘|幺姑姐|姑姐|姑妹|姑姊</t>
         </is>
       </c>
       <c r="J172" t="inlineStr">
@@ -13603,7 +13603,7 @@
       </c>
       <c r="L172" t="inlineStr">
         <is>
-          <t>姑母 | 姑姑|姑媽</t>
+          <t>姑母 | 姑姑|大姑|姑|小姑|老姑|姑媽|姑嬤|姑仔|尕娘|嬢嬢|娘娘|幺姑姐|姑姐|姑妹|姑姊</t>
         </is>
       </c>
       <c r="N172" t="inlineStr">
@@ -13665,7 +13665,7 @@
       </c>
       <c r="H173" t="inlineStr">
         <is>
-          <t>姑父 | 姑丈</t>
+          <t>姑父 | 姑丈|姑夫|恩伯|恩叔|恩爸|姑爹|姑婿|姑郎</t>
         </is>
       </c>
       <c r="J173" t="inlineStr">
@@ -13680,7 +13680,7 @@
       </c>
       <c r="L173" t="inlineStr">
         <is>
-          <t>姑父 | 姑丈</t>
+          <t>姑父 | 姑丈|姑夫|恩伯|恩叔|恩爸|姑爹|姑婿|姑郎</t>
         </is>
       </c>
       <c r="N173" t="inlineStr">
@@ -13742,7 +13742,7 @@
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>叔父 | 叔叔</t>
+          <t>叔父 | 叔叔|小叔|叔|阿叔|依叔|叔仔|叔爸|小爹|小爸|小爸爸|叔爹|仲父|季父</t>
         </is>
       </c>
       <c r="J174" t="inlineStr">
@@ -13757,7 +13757,7 @@
       </c>
       <c r="L174" t="inlineStr">
         <is>
-          <t>叔父 | 叔叔</t>
+          <t>叔父 | 叔叔|小叔|叔|阿叔|依叔|叔仔|叔爸|小爹|小爸|小爸爸|叔爹|仲父|季父</t>
         </is>
       </c>
       <c r="N174" t="inlineStr">
@@ -13819,7 +13819,7 @@
       </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>堂妹</t>
+          <t>堂妹 | 堂細妹</t>
         </is>
       </c>
       <c r="J175" t="inlineStr">
@@ -13834,7 +13834,7 @@
       </c>
       <c r="L175" t="inlineStr">
         <is>
-          <t>堂妹</t>
+          <t>堂妹 | 堂細妹</t>
         </is>
       </c>
       <c r="N175" t="inlineStr">
@@ -13973,7 +13973,7 @@
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>堂外甥婿</t>
+          <t>堂外甥婿 | 堂外甥女婿</t>
         </is>
       </c>
       <c r="J177" t="inlineStr">
@@ -13988,7 +13988,7 @@
       </c>
       <c r="L177" t="inlineStr">
         <is>
-          <t>堂外甥婿</t>
+          <t>堂外甥婿 | 堂外甥女婿</t>
         </is>
       </c>
       <c r="N177" t="inlineStr">
@@ -14127,7 +14127,7 @@
       </c>
       <c r="H179" t="inlineStr">
         <is>
-          <t>堂外甥媳</t>
+          <t>堂外甥媳 | 堂外甥媳婦</t>
         </is>
       </c>
       <c r="J179" t="inlineStr">
@@ -14142,7 +14142,7 @@
       </c>
       <c r="L179" t="inlineStr">
         <is>
-          <t>堂外甥媳</t>
+          <t>堂外甥媳 | 堂外甥媳婦</t>
         </is>
       </c>
       <c r="N179" t="inlineStr">
@@ -14435,7 +14435,7 @@
       </c>
       <c r="H183" t="inlineStr">
         <is>
-          <t>堂姪婿</t>
+          <t>堂姪婿 | 堂姪女婿</t>
         </is>
       </c>
       <c r="J183" t="inlineStr">
@@ -14450,7 +14450,7 @@
       </c>
       <c r="L183" t="inlineStr">
         <is>
-          <t>堂姪婿</t>
+          <t>堂姪婿 | 堂姪女婿</t>
         </is>
       </c>
       <c r="N183" t="inlineStr">
@@ -14512,7 +14512,7 @@
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>堂姪子</t>
+          <t>堂姪子 | 堂姪|再從子</t>
         </is>
       </c>
       <c r="J184" t="inlineStr">
@@ -14527,7 +14527,7 @@
       </c>
       <c r="L184" t="inlineStr">
         <is>
-          <t>堂姪子</t>
+          <t>堂姪子 | 堂姪|再從子</t>
         </is>
       </c>
       <c r="N184" t="inlineStr">
@@ -14589,7 +14589,7 @@
       </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t>堂姪孫子</t>
+          <t>堂姪孫子 | 堂姪孫|再從孫</t>
         </is>
       </c>
       <c r="J185" t="inlineStr">
@@ -14604,7 +14604,7 @@
       </c>
       <c r="L185" t="inlineStr">
         <is>
-          <t>堂姪孫子</t>
+          <t>堂姪孫子 | 堂姪孫|再從孫</t>
         </is>
       </c>
       <c r="N185" t="inlineStr">
@@ -14820,7 +14820,7 @@
       </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t>堂姪媳</t>
+          <t>堂姪媳 | 堂姪媳婦</t>
         </is>
       </c>
       <c r="J188" t="inlineStr">
@@ -14835,7 +14835,7 @@
       </c>
       <c r="L188" t="inlineStr">
         <is>
-          <t>堂姪媳</t>
+          <t>堂姪媳 | 堂姪媳婦</t>
         </is>
       </c>
       <c r="N188" t="inlineStr">
@@ -14897,7 +14897,7 @@
       </c>
       <c r="H189" t="inlineStr">
         <is>
-          <t>堂弟媳</t>
+          <t>堂弟媳 | 堂弟妹|堂弟婦</t>
         </is>
       </c>
       <c r="J189" t="inlineStr">
@@ -14912,7 +14912,7 @@
       </c>
       <c r="L189" t="inlineStr">
         <is>
-          <t>堂弟媳</t>
+          <t>堂弟媳 | 堂弟妹|堂弟婦</t>
         </is>
       </c>
       <c r="N189" t="inlineStr">
@@ -14974,7 +14974,7 @@
       </c>
       <c r="H190" t="inlineStr">
         <is>
-          <t>嬸母 | 嬸嬸</t>
+          <t>嬸母 | 嬸嬸|小嬸|嬸|嬸兒|嬸媽|嬸子|阿嬸|依嬸|叔媽|叔娘|小媽|小媽媽|嬸娘|小娘|家嬸|叔母|仲母|季母|叔婦</t>
         </is>
       </c>
       <c r="J190" t="inlineStr">
@@ -14989,7 +14989,7 @@
       </c>
       <c r="L190" t="inlineStr">
         <is>
-          <t>嬸母 | 嬸嬸</t>
+          <t>嬸母 | 嬸嬸|小嬸|嬸|嬸兒|嬸媽|嬸子|阿嬸|依嬸|叔媽|叔娘|小媽|小媽媽|嬸娘|小娘|家嬸|叔母|仲母|季母|叔婦</t>
         </is>
       </c>
       <c r="N190" t="inlineStr">
@@ -15051,7 +15051,7 @@
       </c>
       <c r="H191" t="inlineStr">
         <is>
-          <t>姑母 | 姑姑|姑媽</t>
+          <t>姑母 | 姑姑|大姑|姑|小姑|老姑|姑媽|姑嬤|姑仔|尕娘|嬢嬢|娘娘|幺姑姐|姑姐|姑妹|姑姊</t>
         </is>
       </c>
       <c r="J191" t="inlineStr">
@@ -15066,7 +15066,7 @@
       </c>
       <c r="L191" t="inlineStr">
         <is>
-          <t>姑母 | 姑姑|姑媽</t>
+          <t>姑母 | 姑姑|大姑|姑|小姑|老姑|姑媽|姑嬤|姑仔|尕娘|嬢嬢|娘娘|幺姑姐|姑姐|姑妹|姑姊</t>
         </is>
       </c>
       <c r="N191" t="inlineStr">
@@ -15128,7 +15128,7 @@
       </c>
       <c r="H192" t="inlineStr">
         <is>
-          <t>姑父 | 姑丈</t>
+          <t>姑父 | 姑丈|姑夫|恩伯|恩叔|恩爸|姑爹|姑婿|姑郎</t>
         </is>
       </c>
       <c r="J192" t="inlineStr">
@@ -15143,7 +15143,7 @@
       </c>
       <c r="L192" t="inlineStr">
         <is>
-          <t>姑父 | 姑丈</t>
+          <t>姑父 | 姑丈|姑夫|恩伯|恩叔|恩爸|姑爹|姑婿|姑郎</t>
         </is>
       </c>
       <c r="N192" t="inlineStr">
@@ -15205,22 +15205,22 @@
       </c>
       <c r="H193" t="inlineStr">
         <is>
+          <t>母親 | 媽媽|老媽|老母親|媽|娘|老母|阿媽|阿母|依媽|阿娘|姆嬤|姆媽|阿毑|媽咪|老乸|母|娘親</t>
+        </is>
+      </c>
+      <c r="J193" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K193" t="inlineStr">
+        <is>
           <t>母親</t>
         </is>
       </c>
-      <c r="J193" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="K193" t="inlineStr">
-        <is>
-          <t>母親</t>
-        </is>
-      </c>
       <c r="L193" t="inlineStr">
         <is>
-          <t>母親</t>
+          <t>母親 | 媽媽|老媽|老母親|媽|娘|老母|阿媽|阿母|依媽|阿娘|姆嬤|姆媽|阿毑|媽咪|老乸|母|娘親</t>
         </is>
       </c>
       <c r="N193" t="inlineStr">
@@ -15282,7 +15282,7 @@
       </c>
       <c r="H194" t="inlineStr">
         <is>
-          <t>外祖父 | 姥爺|外公</t>
+          <t>外祖父 | 姥爺|姥公|舅家爺|姥爹|外公|外爺|尕公|嘎公|嘎爹|嘎嘎爹|嘎爺爺|毑父|毑公|毑爹|毑爺|外大父</t>
         </is>
       </c>
       <c r="J194" t="inlineStr">
@@ -15297,7 +15297,7 @@
       </c>
       <c r="L194" t="inlineStr">
         <is>
-          <t>外祖父 | 姥爺|外公</t>
+          <t>外祖父 | 姥爺|姥公|舅家爺|姥爹|外公|外爺|尕公|嘎公|嘎爹|嘎嘎爹|嘎爺爺|毑父|毑公|毑爹|毑爺|外大父</t>
         </is>
       </c>
       <c r="N194" t="inlineStr">
@@ -15359,7 +15359,7 @@
       </c>
       <c r="H195" t="inlineStr">
         <is>
-          <t>外曾祖父 | 外太爺爺|外太公</t>
+          <t>外曾祖父 | 外太爺爺|外太爺|外太公|外曾祖</t>
         </is>
       </c>
       <c r="J195" t="inlineStr">
@@ -15374,7 +15374,7 @@
       </c>
       <c r="L195" t="inlineStr">
         <is>
-          <t>外曾祖父 | 外太爺爺|外太公</t>
+          <t>外曾祖父 | 外太爺爺|外太爺|外太公|外曾祖</t>
         </is>
       </c>
       <c r="N195" t="inlineStr">
@@ -15590,7 +15590,7 @@
       </c>
       <c r="H198" t="inlineStr">
         <is>
-          <t>外曾祖母 | 外太奶奶|外太婆</t>
+          <t>外曾祖母 | 外太奶奶|外太奶|外太婆</t>
         </is>
       </c>
       <c r="J198" t="inlineStr">
@@ -15605,7 +15605,7 @@
       </c>
       <c r="L198" t="inlineStr">
         <is>
-          <t>外曾祖母 | 外太奶奶|外太婆</t>
+          <t>外曾祖母 | 外太奶奶|外太奶|外太婆</t>
         </is>
       </c>
       <c r="N198" t="inlineStr">
@@ -15821,7 +15821,7 @@
       </c>
       <c r="H201" t="inlineStr">
         <is>
-          <t>伯外祖父 | 伯外公</t>
+          <t>伯外祖父 | 大姥爺|大外爺|伯外公|大外公</t>
         </is>
       </c>
       <c r="J201" t="inlineStr">
@@ -15836,7 +15836,7 @@
       </c>
       <c r="L201" t="inlineStr">
         <is>
-          <t>伯外祖父 | 伯外公</t>
+          <t>伯外祖父 | 大姥爺|大外爺|伯外公|大外公</t>
         </is>
       </c>
       <c r="N201" t="inlineStr">
@@ -15851,12 +15851,12 @@
       </c>
       <c r="P201" t="inlineStr">
         <is>
-          <t>伯外祖父（候選命中：伯外公）</t>
+          <t>伯外祖父（候選命中：大姥爷）</t>
         </is>
       </c>
       <c r="Q201" t="inlineStr">
         <is>
-          <t>可接受簡寫：伯外祖父（候選命中：伯外公）</t>
+          <t>可接受簡寫：伯外祖父（候選命中：大姥爷）</t>
         </is>
       </c>
     </row>
@@ -15975,7 +15975,7 @@
       </c>
       <c r="H203" t="inlineStr">
         <is>
-          <t>堂姨父 | 堂姨丈</t>
+          <t>堂姨父 | 堂姨丈|堂姨夫|堂姨爹|堂姨婿|堂姨郎</t>
         </is>
       </c>
       <c r="J203" t="inlineStr">
@@ -15990,7 +15990,7 @@
       </c>
       <c r="L203" t="inlineStr">
         <is>
-          <t>堂姨父 | 堂姨丈</t>
+          <t>堂姨父 | 堂姨丈|堂姨夫|堂姨爹|堂姨婿|堂姨郎</t>
         </is>
       </c>
       <c r="N203" t="inlineStr">
@@ -16129,7 +16129,7 @@
       </c>
       <c r="H205" t="inlineStr">
         <is>
-          <t>堂舅母 | 堂舅媽</t>
+          <t>堂舅母 | 堂舅媽|堂妗|堂老妗|堂妗子|堂妗妗|堂妗妗兒|堂妗媽|堂舅嬤|堂舅姆|堂阿妗|堂舅娘|堂妗娘|堂舅姆媽|堂舅毑|堂妗母|堂舅妻|堂舅婦</t>
         </is>
       </c>
       <c r="J205" t="inlineStr">
@@ -16144,7 +16144,7 @@
       </c>
       <c r="L205" t="inlineStr">
         <is>
-          <t>堂舅母 | 堂舅媽</t>
+          <t>堂舅母 | 堂舅媽|堂妗|堂老妗|堂妗子|堂妗妗|堂妗妗兒|堂妗媽|堂舅嬤|堂舅姆|堂阿妗|堂舅娘|堂妗娘|堂舅姆媽|堂舅毑|堂妗母|堂舅妻|堂舅婦</t>
         </is>
       </c>
       <c r="N205" t="inlineStr">
@@ -16206,7 +16206,7 @@
       </c>
       <c r="H206" t="inlineStr">
         <is>
-          <t>伯外祖母 | 伯外婆</t>
+          <t>伯外祖母 | 大姥姥|伯外婆|大外婆</t>
         </is>
       </c>
       <c r="J206" t="inlineStr">
@@ -16221,7 +16221,7 @@
       </c>
       <c r="L206" t="inlineStr">
         <is>
-          <t>伯外祖母 | 伯外婆</t>
+          <t>伯外祖母 | 大姥姥|伯外婆|大外婆</t>
         </is>
       </c>
       <c r="N206" t="inlineStr">
@@ -16236,12 +16236,12 @@
       </c>
       <c r="P206" t="inlineStr">
         <is>
-          <t>伯外祖母（候選命中：伯外婆）</t>
+          <t>伯外祖母（候選命中：大姥姥）</t>
         </is>
       </c>
       <c r="Q206" t="inlineStr">
         <is>
-          <t>可接受簡寫：伯外祖母（候選命中：伯外婆）</t>
+          <t>可接受簡寫：伯外祖母（候選命中：大姥姥）</t>
         </is>
       </c>
     </row>
@@ -16360,7 +16360,7 @@
       </c>
       <c r="H208" t="inlineStr">
         <is>
-          <t>姑外祖父 | 姑外公</t>
+          <t>姑外祖父 | 姑外公|外姑丈公|恩爹</t>
         </is>
       </c>
       <c r="J208" t="inlineStr">
@@ -16375,7 +16375,7 @@
       </c>
       <c r="L208" t="inlineStr">
         <is>
-          <t>姑外祖父 | 姑外公</t>
+          <t>姑外祖父 | 姑外公|外姑丈公|恩爹</t>
         </is>
       </c>
       <c r="N208" t="inlineStr">
@@ -16437,7 +16437,7 @@
       </c>
       <c r="H209" t="inlineStr">
         <is>
-          <t>叔外祖父 | 叔外公</t>
+          <t>叔外祖父 | 小姥爺|小外爺|叔外公|小外公</t>
         </is>
       </c>
       <c r="J209" t="inlineStr">
@@ -16452,7 +16452,7 @@
       </c>
       <c r="L209" t="inlineStr">
         <is>
-          <t>叔外祖父 | 叔外公</t>
+          <t>叔外祖父 | 小姥爺|小外爺|叔外公|小外公</t>
         </is>
       </c>
       <c r="N209" t="inlineStr">
@@ -16467,12 +16467,12 @@
       </c>
       <c r="P209" t="inlineStr">
         <is>
-          <t>叔外祖父（候選命中：叔外公）</t>
+          <t>叔外祖父（候選命中：小姥爷）</t>
         </is>
       </c>
       <c r="Q209" t="inlineStr">
         <is>
-          <t>可接受簡寫：叔外祖父（候選命中：叔外公）</t>
+          <t>可接受簡寫：叔外祖父（候選命中：小姥爷）</t>
         </is>
       </c>
     </row>
@@ -16591,7 +16591,7 @@
       </c>
       <c r="H211" t="inlineStr">
         <is>
-          <t>堂姨父 | 堂姨丈</t>
+          <t>堂姨父 | 堂姨丈|堂姨夫|堂姨爹|堂姨婿|堂姨郎</t>
         </is>
       </c>
       <c r="J211" t="inlineStr">
@@ -16606,7 +16606,7 @@
       </c>
       <c r="L211" t="inlineStr">
         <is>
-          <t>堂姨父 | 堂姨丈</t>
+          <t>堂姨父 | 堂姨丈|堂姨夫|堂姨爹|堂姨婿|堂姨郎</t>
         </is>
       </c>
       <c r="N211" t="inlineStr">
@@ -16745,7 +16745,7 @@
       </c>
       <c r="H213" t="inlineStr">
         <is>
-          <t>堂舅母 | 堂舅媽</t>
+          <t>堂舅母 | 堂舅媽|堂妗|堂老妗|堂妗子|堂妗妗|堂妗妗兒|堂妗媽|堂舅嬤|堂舅姆|堂阿妗|堂舅娘|堂妗娘|堂舅姆媽|堂舅毑|堂妗母|堂舅妻|堂舅婦</t>
         </is>
       </c>
       <c r="J213" t="inlineStr">
@@ -16760,7 +16760,7 @@
       </c>
       <c r="L213" t="inlineStr">
         <is>
-          <t>堂舅母 | 堂舅媽</t>
+          <t>堂舅母 | 堂舅媽|堂妗|堂老妗|堂妗子|堂妗妗|堂妗妗兒|堂妗媽|堂舅嬤|堂舅姆|堂阿妗|堂舅娘|堂妗娘|堂舅姆媽|堂舅毑|堂妗母|堂舅妻|堂舅婦</t>
         </is>
       </c>
       <c r="N213" t="inlineStr">
@@ -16822,7 +16822,7 @@
       </c>
       <c r="H214" t="inlineStr">
         <is>
-          <t>叔外祖母 | 叔外婆</t>
+          <t>叔外祖母 | 小姥姥|嬸姥姥|叔外婆|小外婆</t>
         </is>
       </c>
       <c r="J214" t="inlineStr">
@@ -16837,7 +16837,7 @@
       </c>
       <c r="L214" t="inlineStr">
         <is>
-          <t>叔外祖母 | 叔外婆</t>
+          <t>叔外祖母 | 小姥姥|嬸姥姥|叔外婆|小外婆</t>
         </is>
       </c>
       <c r="N214" t="inlineStr">
@@ -16852,12 +16852,12 @@
       </c>
       <c r="P214" t="inlineStr">
         <is>
-          <t>叔外祖母（候選命中：叔外婆）</t>
+          <t>叔外祖母（候選命中：小姥姥）</t>
         </is>
       </c>
       <c r="Q214" t="inlineStr">
         <is>
-          <t>可接受簡寫：叔外祖母（候選命中：叔外婆）</t>
+          <t>可接受簡寫：叔外祖母（候選命中：小姥姥）</t>
         </is>
       </c>
     </row>
@@ -16976,7 +16976,7 @@
       </c>
       <c r="H216" t="inlineStr">
         <is>
-          <t>姑外祖父 | 姑外公</t>
+          <t>姑外祖父 | 姑外公|外姑丈公|恩爹</t>
         </is>
       </c>
       <c r="J216" t="inlineStr">
@@ -16991,7 +16991,7 @@
       </c>
       <c r="L216" t="inlineStr">
         <is>
-          <t>姑外祖父 | 姑外公</t>
+          <t>姑外祖父 | 姑外公|外姑丈公|恩爹</t>
         </is>
       </c>
       <c r="N216" t="inlineStr">
@@ -17053,7 +17053,7 @@
       </c>
       <c r="H217" t="inlineStr">
         <is>
-          <t>外祖母 | 姥姥|外婆</t>
+          <t>外祖母 | 姥姥|外奶|姥婆|舅家婆|姥娘|姥|外婆|外嬤|尕婆|嘎嘎|嘎婆|嘎嘎婆|嘎奶奶|阿婆|好婆|毑母|毑婆|毑娘|毑毑|嫲嫲|外大母</t>
         </is>
       </c>
       <c r="J217" t="inlineStr">
@@ -17068,7 +17068,7 @@
       </c>
       <c r="L217" t="inlineStr">
         <is>
-          <t>外祖母 | 姥姥|外婆</t>
+          <t>外祖母 | 姥姥|外奶|姥婆|舅家婆|姥娘|姥|外婆|外嬤|尕婆|嘎嘎|嘎婆|嘎嘎婆|嘎奶奶|阿婆|好婆|毑母|毑婆|毑娘|毑毑|嫲嫲|外大母</t>
         </is>
       </c>
       <c r="N217" t="inlineStr">
@@ -17130,7 +17130,7 @@
       </c>
       <c r="H218" t="inlineStr">
         <is>
-          <t>外曾外祖父</t>
+          <t>外曾外祖父 | 外太姥爺|曾毑父|外曾外祖</t>
         </is>
       </c>
       <c r="J218" t="inlineStr">
@@ -17145,7 +17145,7 @@
       </c>
       <c r="L218" t="inlineStr">
         <is>
-          <t>外曾外祖父</t>
+          <t>外曾外祖父 | 外太姥爺|曾毑父|外曾外祖</t>
         </is>
       </c>
       <c r="N218" t="inlineStr">
@@ -17361,7 +17361,7 @@
       </c>
       <c r="H221" t="inlineStr">
         <is>
-          <t>外曾外祖母</t>
+          <t>外曾外祖母 | 外太姥姥|曾毑母</t>
         </is>
       </c>
       <c r="J221" t="inlineStr">
@@ -17376,7 +17376,7 @@
       </c>
       <c r="L221" t="inlineStr">
         <is>
-          <t>外曾外祖母</t>
+          <t>外曾外祖母 | 外太姥姥|曾毑母</t>
         </is>
       </c>
       <c r="N221" t="inlineStr">
@@ -17669,7 +17669,7 @@
       </c>
       <c r="H225" t="inlineStr">
         <is>
-          <t>舅外祖母 | 舅外婆</t>
+          <t>舅外祖母 | 妗姥姥|妗姥娘|妗姥|舅外婆</t>
         </is>
       </c>
       <c r="J225" t="inlineStr">
@@ -17684,7 +17684,7 @@
       </c>
       <c r="L225" t="inlineStr">
         <is>
-          <t>舅外祖母 | 舅外婆</t>
+          <t>舅外祖母 | 妗姥姥|妗姥娘|妗姥|舅外婆</t>
         </is>
       </c>
       <c r="N225" t="inlineStr">
@@ -17699,12 +17699,12 @@
       </c>
       <c r="P225" t="inlineStr">
         <is>
-          <t>舅外祖母（候選命中：舅外婆）</t>
+          <t>舅外祖母（候選命中：妗姥姥）</t>
         </is>
       </c>
       <c r="Q225" t="inlineStr">
         <is>
-          <t>可接受簡寫：舅外祖母（候選命中：舅外婆）</t>
+          <t>可接受簡寫：舅外祖母（候選命中：妗姥姥）</t>
         </is>
       </c>
     </row>
@@ -17823,7 +17823,7 @@
       </c>
       <c r="H227" t="inlineStr">
         <is>
-          <t>姨外祖父 | 姨外公</t>
+          <t>姨外祖父 | 姨外公|外姨丈公</t>
         </is>
       </c>
       <c r="J227" t="inlineStr">
@@ -17838,7 +17838,7 @@
       </c>
       <c r="L227" t="inlineStr">
         <is>
-          <t>姨外祖父 | 姨外公</t>
+          <t>姨外祖父 | 姨外公|外姨丈公</t>
         </is>
       </c>
       <c r="N227" t="inlineStr">
@@ -17977,7 +17977,7 @@
       </c>
       <c r="H229" t="inlineStr">
         <is>
-          <t>舅外祖母 | 舅外婆</t>
+          <t>舅外祖母 | 妗姥姥|妗姥娘|妗姥|舅外婆</t>
         </is>
       </c>
       <c r="J229" t="inlineStr">
@@ -17992,7 +17992,7 @@
       </c>
       <c r="L229" t="inlineStr">
         <is>
-          <t>舅外祖母 | 舅外婆</t>
+          <t>舅外祖母 | 妗姥姥|妗姥娘|妗姥|舅外婆</t>
         </is>
       </c>
       <c r="N229" t="inlineStr">
@@ -18007,12 +18007,12 @@
       </c>
       <c r="P229" t="inlineStr">
         <is>
-          <t>舅外祖母（候選命中：舅外婆）</t>
+          <t>舅外祖母（候選命中：妗姥姥）</t>
         </is>
       </c>
       <c r="Q229" t="inlineStr">
         <is>
-          <t>可接受簡寫：舅外祖母（候選命中：舅外婆）</t>
+          <t>可接受簡寫：舅外祖母（候選命中：妗姥姥）</t>
         </is>
       </c>
     </row>
@@ -18131,7 +18131,7 @@
       </c>
       <c r="H231" t="inlineStr">
         <is>
-          <t>姨外祖父 | 姨外公</t>
+          <t>姨外祖父 | 姨外公|外姨丈公</t>
         </is>
       </c>
       <c r="J231" t="inlineStr">
@@ -18146,7 +18146,7 @@
       </c>
       <c r="L231" t="inlineStr">
         <is>
-          <t>姨外祖父 | 姨外公</t>
+          <t>姨外祖父 | 姨外公|外姨丈公</t>
         </is>
       </c>
       <c r="N231" t="inlineStr">
@@ -18208,7 +18208,7 @@
       </c>
       <c r="H232" t="inlineStr">
         <is>
-          <t>舅父 | 舅舅</t>
+          <t>舅父 | 舅舅|大舅|大舅舅|舅|小舅|小舅舅|老舅|母舅|阿舅|舅仔|尕阿舅|舅爸|舅爹|娘舅|元舅|舅台</t>
         </is>
       </c>
       <c r="J232" t="inlineStr">
@@ -18223,7 +18223,7 @@
       </c>
       <c r="L232" t="inlineStr">
         <is>
-          <t>舅父 | 舅舅</t>
+          <t>舅父 | 舅舅|大舅|大舅舅|舅|小舅|小舅舅|老舅|母舅|阿舅|舅仔|尕阿舅|舅爸|舅爹|娘舅|元舅|舅台</t>
         </is>
       </c>
       <c r="N232" t="inlineStr">
@@ -18285,7 +18285,7 @@
       </c>
       <c r="H233" t="inlineStr">
         <is>
-          <t>舅母 | 舅媽</t>
+          <t>舅母 | 舅媽|妗|老妗|妗子|妗妗|妗妗兒|妗媽|舅嬤|舅姆|阿妗|舅娘|妗娘|舅姆媽|舅毑|妗母|舅妻|舅婦</t>
         </is>
       </c>
       <c r="J233" t="inlineStr">
@@ -18300,7 +18300,7 @@
       </c>
       <c r="L233" t="inlineStr">
         <is>
-          <t>舅母 | 舅媽</t>
+          <t>舅母 | 舅媽|妗|老妗|妗子|妗妗|妗妗兒|妗媽|舅嬤|舅姆|阿妗|舅娘|妗娘|舅姆媽|舅毑|妗母|舅妻|舅婦</t>
         </is>
       </c>
       <c r="N233" t="inlineStr">
@@ -18362,7 +18362,7 @@
       </c>
       <c r="H234" t="inlineStr">
         <is>
-          <t>姨母 | 阿姨|姨媽</t>
+          <t>姨母 | 阿姨|大姨|姨姨|姨|小姨|老姨|姨媽|姨嬤|姨仔|嬢嬢|姨娘|從母</t>
         </is>
       </c>
       <c r="J234" t="inlineStr">
@@ -18377,7 +18377,7 @@
       </c>
       <c r="L234" t="inlineStr">
         <is>
-          <t>姨母 | 阿姨|姨媽</t>
+          <t>姨母 | 阿姨|大姨|姨姨|姨|小姨|老姨|姨媽|姨嬤|姨仔|嬢嬢|姨娘|從母</t>
         </is>
       </c>
       <c r="N234" t="inlineStr">
@@ -18439,7 +18439,7 @@
       </c>
       <c r="H235" t="inlineStr">
         <is>
-          <t>姨父 | 姨丈</t>
+          <t>姨父 | 姨丈|姨夫|姨爹|姨婿|姨郎</t>
         </is>
       </c>
       <c r="J235" t="inlineStr">
@@ -18454,7 +18454,7 @@
       </c>
       <c r="L235" t="inlineStr">
         <is>
-          <t>姨父 | 姨丈</t>
+          <t>姨父 | 姨丈|姨夫|姨爹|姨婿|姨郎</t>
         </is>
       </c>
       <c r="N235" t="inlineStr">
@@ -18516,7 +18516,7 @@
       </c>
       <c r="H236" t="inlineStr">
         <is>
-          <t>舅父 | 舅舅</t>
+          <t>舅父 | 舅舅|大舅|大舅舅|舅|小舅|小舅舅|老舅|母舅|阿舅|舅仔|尕阿舅|舅爸|舅爹|娘舅|元舅|舅台</t>
         </is>
       </c>
       <c r="J236" t="inlineStr">
@@ -18531,7 +18531,7 @@
       </c>
       <c r="L236" t="inlineStr">
         <is>
-          <t>舅父 | 舅舅</t>
+          <t>舅父 | 舅舅|大舅|大舅舅|舅|小舅|小舅舅|老舅|母舅|阿舅|舅仔|尕阿舅|舅爸|舅爹|娘舅|元舅|舅台</t>
         </is>
       </c>
       <c r="N236" t="inlineStr">
@@ -18593,7 +18593,7 @@
       </c>
       <c r="H237" t="inlineStr">
         <is>
-          <t>舅母 | 舅媽</t>
+          <t>舅母 | 舅媽|妗|老妗|妗子|妗妗|妗妗兒|妗媽|舅嬤|舅姆|阿妗|舅娘|妗娘|舅姆媽|舅毑|妗母|舅妻|舅婦</t>
         </is>
       </c>
       <c r="J237" t="inlineStr">
@@ -18608,7 +18608,7 @@
       </c>
       <c r="L237" t="inlineStr">
         <is>
-          <t>舅母 | 舅媽</t>
+          <t>舅母 | 舅媽|妗|老妗|妗子|妗妗|妗妗兒|妗媽|舅嬤|舅姆|阿妗|舅娘|妗娘|舅姆媽|舅毑|妗母|舅妻|舅婦</t>
         </is>
       </c>
       <c r="N237" t="inlineStr">
@@ -18670,7 +18670,7 @@
       </c>
       <c r="H238" t="inlineStr">
         <is>
-          <t>姨母 | 阿姨|姨媽</t>
+          <t>姨母 | 阿姨|大姨|姨姨|姨|小姨|老姨|姨媽|姨嬤|姨仔|嬢嬢|姨娘|從母</t>
         </is>
       </c>
       <c r="J238" t="inlineStr">
@@ -18685,7 +18685,7 @@
       </c>
       <c r="L238" t="inlineStr">
         <is>
-          <t>姨母 | 阿姨|姨媽</t>
+          <t>姨母 | 阿姨|大姨|姨姨|姨|小姨|老姨|姨媽|姨嬤|姨仔|嬢嬢|姨娘|從母</t>
         </is>
       </c>
       <c r="N238" t="inlineStr">
@@ -18747,7 +18747,7 @@
       </c>
       <c r="H239" t="inlineStr">
         <is>
-          <t>姨父 | 姨丈</t>
+          <t>姨父 | 姨丈|姨夫|姨爹|姨婿|姨郎</t>
         </is>
       </c>
       <c r="J239" t="inlineStr">
@@ -18762,7 +18762,7 @@
       </c>
       <c r="L239" t="inlineStr">
         <is>
-          <t>姨父 | 姨丈</t>
+          <t>姨父 | 姨丈|姨夫|姨爹|姨婿|姨郎</t>
         </is>
       </c>
       <c r="N239" t="inlineStr">
@@ -18824,22 +18824,22 @@
       </c>
       <c r="H240" t="inlineStr">
         <is>
+          <t>哥哥 | 哥|親哥|老哥|依哥|阿哥|大佬|胞兄|兄台|家兄|兄長</t>
+        </is>
+      </c>
+      <c r="J240" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K240" t="inlineStr">
+        <is>
           <t>哥哥</t>
         </is>
       </c>
-      <c r="J240" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="K240" t="inlineStr">
-        <is>
-          <t>哥哥</t>
-        </is>
-      </c>
       <c r="L240" t="inlineStr">
         <is>
-          <t>哥哥</t>
+          <t>哥哥 | 哥|親哥|老哥|依哥|阿哥|大佬|胞兄|兄台|家兄|兄長</t>
         </is>
       </c>
       <c r="N240" t="inlineStr">
@@ -18901,7 +18901,7 @@
       </c>
       <c r="H241" t="inlineStr">
         <is>
-          <t>姪女</t>
+          <t>姪女 | 姪女兒|姪丫頭|姪閨女|姪囡|兄女</t>
         </is>
       </c>
       <c r="J241" t="inlineStr">
@@ -18916,7 +18916,7 @@
       </c>
       <c r="L241" t="inlineStr">
         <is>
-          <t>姪女</t>
+          <t>姪女 | 姪女兒|姪丫頭|姪閨女|姪囡|兄女</t>
         </is>
       </c>
       <c r="N241" t="inlineStr">
@@ -18978,7 +18978,7 @@
       </c>
       <c r="H242" t="inlineStr">
         <is>
-          <t>姪女婿</t>
+          <t>姪女婿 | 姪婿</t>
         </is>
       </c>
       <c r="J242" t="inlineStr">
@@ -18993,7 +18993,7 @@
       </c>
       <c r="L242" t="inlineStr">
         <is>
-          <t>姪女婿</t>
+          <t>姪女婿 | 姪婿</t>
         </is>
       </c>
       <c r="N242" t="inlineStr">
@@ -19055,7 +19055,7 @@
       </c>
       <c r="H243" t="inlineStr">
         <is>
-          <t>姪子</t>
+          <t>姪子 | 親姪|姪兒|姪|姪小子|老姪|姪仔|阿姪|兄子|姪男|嫡姪</t>
         </is>
       </c>
       <c r="J243" t="inlineStr">
@@ -19070,7 +19070,7 @@
       </c>
       <c r="L243" t="inlineStr">
         <is>
-          <t>姪子</t>
+          <t>姪子 | 親姪|姪兒|姪|姪小子|老姪|姪仔|阿姪|兄子|姪男|嫡姪</t>
         </is>
       </c>
       <c r="N243" t="inlineStr">
@@ -19132,7 +19132,7 @@
       </c>
       <c r="H244" t="inlineStr">
         <is>
-          <t>姪媳婦</t>
+          <t>姪媳婦 | 姪媳|姪婦</t>
         </is>
       </c>
       <c r="J244" t="inlineStr">
@@ -19147,7 +19147,7 @@
       </c>
       <c r="L244" t="inlineStr">
         <is>
-          <t>姪媳婦</t>
+          <t>姪媳婦 | 姪媳|姪婦</t>
         </is>
       </c>
       <c r="N244" t="inlineStr">
@@ -19209,7 +19209,7 @@
       </c>
       <c r="H245" t="inlineStr">
         <is>
-          <t>嫂嫂 | 嫂子</t>
+          <t>嫂嫂 | 嫂子|嫂|阿嫂|家嫂|兄婦|兄妻</t>
         </is>
       </c>
       <c r="J245" t="inlineStr">
@@ -19224,7 +19224,7 @@
       </c>
       <c r="L245" t="inlineStr">
         <is>
-          <t>嫂嫂 | 嫂子</t>
+          <t>嫂嫂 | 嫂子|嫂|阿嫂|家嫂|兄婦|兄妻</t>
         </is>
       </c>
       <c r="N245" t="inlineStr">
@@ -19286,22 +19286,22 @@
       </c>
       <c r="H246" t="inlineStr">
         <is>
+          <t>姐姐 | 姐|親姐|老姐|依姐|姊仔|阿姐|家姐|胞姐|姊台</t>
+        </is>
+      </c>
+      <c r="J246" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K246" t="inlineStr">
+        <is>
           <t>姐姐</t>
         </is>
       </c>
-      <c r="J246" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="K246" t="inlineStr">
-        <is>
-          <t>姐姐</t>
-        </is>
-      </c>
       <c r="L246" t="inlineStr">
         <is>
-          <t>姐姐</t>
+          <t>姐姐 | 姐|親姐|老姐|依姐|姊仔|阿姐|家姐|胞姐|姊台</t>
         </is>
       </c>
       <c r="N246" t="inlineStr">
@@ -19363,7 +19363,7 @@
       </c>
       <c r="H247" t="inlineStr">
         <is>
-          <t>外甥女</t>
+          <t>外甥女 | 甥女兒|甥閨女|甥囡|甥女</t>
         </is>
       </c>
       <c r="J247" t="inlineStr">
@@ -19378,7 +19378,7 @@
       </c>
       <c r="L247" t="inlineStr">
         <is>
-          <t>外甥女</t>
+          <t>外甥女 | 甥女兒|甥閨女|甥囡|甥女</t>
         </is>
       </c>
       <c r="N247" t="inlineStr">
@@ -19440,7 +19440,7 @@
       </c>
       <c r="H248" t="inlineStr">
         <is>
-          <t>外甥婿</t>
+          <t>外甥婿 | 甥女婿|甥婿</t>
         </is>
       </c>
       <c r="J248" t="inlineStr">
@@ -19455,7 +19455,7 @@
       </c>
       <c r="L248" t="inlineStr">
         <is>
-          <t>外甥婿</t>
+          <t>外甥婿 | 甥女婿|甥婿</t>
         </is>
       </c>
       <c r="N248" t="inlineStr">
@@ -19517,7 +19517,7 @@
       </c>
       <c r="H249" t="inlineStr">
         <is>
-          <t>外甥</t>
+          <t>外甥 | 甥兒|甥仔|甥子|甥男|甥</t>
         </is>
       </c>
       <c r="J249" t="inlineStr">
@@ -19532,7 +19532,7 @@
       </c>
       <c r="L249" t="inlineStr">
         <is>
-          <t>外甥</t>
+          <t>外甥 | 甥兒|甥仔|甥子|甥男|甥</t>
         </is>
       </c>
       <c r="N249" t="inlineStr">
@@ -19594,7 +19594,7 @@
       </c>
       <c r="H250" t="inlineStr">
         <is>
-          <t>外甥孫女</t>
+          <t>外甥孫女 | 甥孫女|遠甥女|彌甥女</t>
         </is>
       </c>
       <c r="J250" t="inlineStr">
@@ -19609,7 +19609,7 @@
       </c>
       <c r="L250" t="inlineStr">
         <is>
-          <t>外甥孫女</t>
+          <t>外甥孫女 | 甥孫女|遠甥女|彌甥女</t>
         </is>
       </c>
       <c r="N250" t="inlineStr">
@@ -19671,7 +19671,7 @@
       </c>
       <c r="H251" t="inlineStr">
         <is>
-          <t>外甥孫</t>
+          <t>外甥孫 | 甥孫|遠甥|彌甥</t>
         </is>
       </c>
       <c r="J251" t="inlineStr">
@@ -19686,7 +19686,7 @@
       </c>
       <c r="L251" t="inlineStr">
         <is>
-          <t>外甥孫</t>
+          <t>外甥孫 | 甥孫|遠甥|彌甥</t>
         </is>
       </c>
       <c r="N251" t="inlineStr">
@@ -19748,7 +19748,7 @@
       </c>
       <c r="H252" t="inlineStr">
         <is>
-          <t>外甥媳</t>
+          <t>外甥媳 | 甥媳婦|甥媳|甥婦</t>
         </is>
       </c>
       <c r="J252" t="inlineStr">
@@ -19763,7 +19763,7 @@
       </c>
       <c r="L252" t="inlineStr">
         <is>
-          <t>外甥媳</t>
+          <t>外甥媳 | 甥媳婦|甥媳|甥婦</t>
         </is>
       </c>
       <c r="N252" t="inlineStr">
@@ -19825,7 +19825,7 @@
       </c>
       <c r="H253" t="inlineStr">
         <is>
-          <t>姐夫 | 連襟</t>
+          <t>姐夫 | 姐丈|姐夫哥|姐婿</t>
         </is>
       </c>
       <c r="J253" t="inlineStr">
@@ -19840,7 +19840,7 @@
       </c>
       <c r="L253" t="inlineStr">
         <is>
-          <t>姐夫 | 連襟</t>
+          <t>姐夫 | 姐丈|姐夫哥|姐婿</t>
         </is>
       </c>
       <c r="N253" t="inlineStr">
@@ -19902,22 +19902,22 @@
       </c>
       <c r="H254" t="inlineStr">
         <is>
+          <t>兒子 | 小子|後生|囝男|囝兒|囝|娃子|伢子|囝囝|仔|阿仔|仔仔|男兒|息男|兒|子</t>
+        </is>
+      </c>
+      <c r="J254" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K254" t="inlineStr">
+        <is>
           <t>兒子</t>
         </is>
       </c>
-      <c r="J254" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="K254" t="inlineStr">
-        <is>
-          <t>兒子</t>
-        </is>
-      </c>
       <c r="L254" t="inlineStr">
         <is>
-          <t>兒子</t>
+          <t>兒子 | 小子|後生|囝男|囝兒|囝|娃子|伢子|囝囝|仔|阿仔|仔仔|男兒|息男|兒|子</t>
         </is>
       </c>
       <c r="N254" t="inlineStr">
@@ -19979,7 +19979,7 @@
       </c>
       <c r="H255" t="inlineStr">
         <is>
-          <t>孫女</t>
+          <t>孫女 | 孫女兒|孫囡|孫囡兒|女孫</t>
         </is>
       </c>
       <c r="J255" t="inlineStr">
@@ -19994,7 +19994,7 @@
       </c>
       <c r="L255" t="inlineStr">
         <is>
-          <t>孫女</t>
+          <t>孫女 | 孫女兒|孫囡|孫囡兒|女孫</t>
         </is>
       </c>
       <c r="N255" t="inlineStr">
@@ -20518,7 +20518,7 @@
       </c>
       <c r="H262" t="inlineStr">
         <is>
-          <t>曾外孫子</t>
+          <t>曾外孫子 | 曾外孫</t>
         </is>
       </c>
       <c r="J262" t="inlineStr">
@@ -20533,7 +20533,7 @@
       </c>
       <c r="L262" t="inlineStr">
         <is>
-          <t>曾外孫子</t>
+          <t>曾外孫子 | 曾外孫</t>
         </is>
       </c>
       <c r="N262" t="inlineStr">
@@ -20595,7 +20595,7 @@
       </c>
       <c r="H263" t="inlineStr">
         <is>
-          <t>玄孫女</t>
+          <t>玄孫女 | 元孫女</t>
         </is>
       </c>
       <c r="J263" t="inlineStr">
@@ -20610,7 +20610,7 @@
       </c>
       <c r="L263" t="inlineStr">
         <is>
-          <t>玄孫女</t>
+          <t>玄孫女 | 元孫女</t>
         </is>
       </c>
       <c r="N263" t="inlineStr">
@@ -20672,7 +20672,7 @@
       </c>
       <c r="H264" t="inlineStr">
         <is>
-          <t>玄孫婿</t>
+          <t>玄孫婿 | 玄孫女婿</t>
         </is>
       </c>
       <c r="J264" t="inlineStr">
@@ -20687,7 +20687,7 @@
       </c>
       <c r="L264" t="inlineStr">
         <is>
-          <t>玄孫婿</t>
+          <t>玄孫婿 | 玄孫女婿</t>
         </is>
       </c>
       <c r="N264" t="inlineStr">
@@ -20749,7 +20749,7 @@
       </c>
       <c r="H265" t="inlineStr">
         <is>
-          <t>玄孫子</t>
+          <t>玄孫子 | 重重孫|玄孫|元孫</t>
         </is>
       </c>
       <c r="J265" t="inlineStr">
@@ -20764,7 +20764,7 @@
       </c>
       <c r="L265" t="inlineStr">
         <is>
-          <t>玄孫子</t>
+          <t>玄孫子 | 重重孫|玄孫|元孫</t>
         </is>
       </c>
       <c r="N265" t="inlineStr">
@@ -20826,7 +20826,7 @@
       </c>
       <c r="H266" t="inlineStr">
         <is>
-          <t>玄孫媳</t>
+          <t>玄孫媳 | 玄孫媳婦</t>
         </is>
       </c>
       <c r="J266" t="inlineStr">
@@ -20841,7 +20841,7 @@
       </c>
       <c r="L266" t="inlineStr">
         <is>
-          <t>玄孫媳</t>
+          <t>玄孫媳 | 玄孫媳婦</t>
         </is>
       </c>
       <c r="N266" t="inlineStr">
@@ -20980,7 +20980,7 @@
       </c>
       <c r="H268" t="inlineStr">
         <is>
-          <t>孫婿</t>
+          <t>孫婿 | 孫女婿</t>
         </is>
       </c>
       <c r="J268" t="inlineStr">
@@ -20995,7 +20995,7 @@
       </c>
       <c r="L268" t="inlineStr">
         <is>
-          <t>孫婿</t>
+          <t>孫婿 | 孫女婿</t>
         </is>
       </c>
       <c r="N268" t="inlineStr">
@@ -21057,7 +21057,7 @@
       </c>
       <c r="H269" t="inlineStr">
         <is>
-          <t>孫子</t>
+          <t>孫子 | 孫兒|孫仔|孫囝|孫娃子|孫伢子|孫男|嗣孫</t>
         </is>
       </c>
       <c r="J269" t="inlineStr">
@@ -21072,7 +21072,7 @@
       </c>
       <c r="L269" t="inlineStr">
         <is>
-          <t>孫子</t>
+          <t>孫子 | 孫兒|孫仔|孫囝|孫娃子|孫伢子|孫男|嗣孫</t>
         </is>
       </c>
       <c r="N269" t="inlineStr">
@@ -21134,7 +21134,7 @@
       </c>
       <c r="H270" t="inlineStr">
         <is>
-          <t>曾孫女</t>
+          <t>曾孫女 | 重孫女</t>
         </is>
       </c>
       <c r="J270" t="inlineStr">
@@ -21149,7 +21149,7 @@
       </c>
       <c r="L270" t="inlineStr">
         <is>
-          <t>曾孫女</t>
+          <t>曾孫女 | 重孫女</t>
         </is>
       </c>
       <c r="N270" t="inlineStr">
@@ -21519,7 +21519,7 @@
       </c>
       <c r="H275" t="inlineStr">
         <is>
-          <t>曾孫婿</t>
+          <t>曾孫婿 | 曾孫女婿</t>
         </is>
       </c>
       <c r="J275" t="inlineStr">
@@ -21534,7 +21534,7 @@
       </c>
       <c r="L275" t="inlineStr">
         <is>
-          <t>曾孫婿</t>
+          <t>曾孫婿 | 曾孫女婿</t>
         </is>
       </c>
       <c r="N275" t="inlineStr">
@@ -21596,7 +21596,7 @@
       </c>
       <c r="H276" t="inlineStr">
         <is>
-          <t>曾孫子</t>
+          <t>曾孫子 | 重孫|重孫子|曾孫</t>
         </is>
       </c>
       <c r="J276" t="inlineStr">
@@ -21611,7 +21611,7 @@
       </c>
       <c r="L276" t="inlineStr">
         <is>
-          <t>曾孫子</t>
+          <t>曾孫子 | 重孫|重孫子|曾孫</t>
         </is>
       </c>
       <c r="N276" t="inlineStr">
@@ -21673,7 +21673,7 @@
       </c>
       <c r="H277" t="inlineStr">
         <is>
-          <t>玄孫女</t>
+          <t>玄孫女 | 元孫女</t>
         </is>
       </c>
       <c r="J277" t="inlineStr">
@@ -21688,7 +21688,7 @@
       </c>
       <c r="L277" t="inlineStr">
         <is>
-          <t>玄孫女</t>
+          <t>玄孫女 | 元孫女</t>
         </is>
       </c>
       <c r="N277" t="inlineStr">
@@ -22058,7 +22058,7 @@
       </c>
       <c r="H282" t="inlineStr">
         <is>
-          <t>玄孫婿</t>
+          <t>玄孫婿 | 玄孫女婿</t>
         </is>
       </c>
       <c r="J282" t="inlineStr">
@@ -22073,7 +22073,7 @@
       </c>
       <c r="L282" t="inlineStr">
         <is>
-          <t>玄孫婿</t>
+          <t>玄孫婿 | 玄孫女婿</t>
         </is>
       </c>
       <c r="N282" t="inlineStr">
@@ -22135,7 +22135,7 @@
       </c>
       <c r="H283" t="inlineStr">
         <is>
-          <t>玄孫子</t>
+          <t>玄孫子 | 重重孫|玄孫|元孫</t>
         </is>
       </c>
       <c r="J283" t="inlineStr">
@@ -22150,7 +22150,7 @@
       </c>
       <c r="L283" t="inlineStr">
         <is>
-          <t>玄孫子</t>
+          <t>玄孫子 | 重重孫|玄孫|元孫</t>
         </is>
       </c>
       <c r="N283" t="inlineStr">
@@ -22597,7 +22597,7 @@
       </c>
       <c r="H289" t="inlineStr">
         <is>
-          <t>來孫婿</t>
+          <t>來孫婿 | 來孫女婿</t>
         </is>
       </c>
       <c r="J289" t="inlineStr">
@@ -22612,7 +22612,7 @@
       </c>
       <c r="L289" t="inlineStr">
         <is>
-          <t>來孫婿</t>
+          <t>來孫婿 | 來孫女婿</t>
         </is>
       </c>
       <c r="N289" t="inlineStr">
@@ -22674,7 +22674,7 @@
       </c>
       <c r="H290" t="inlineStr">
         <is>
-          <t>來孫子</t>
+          <t>來孫子 | 來孫</t>
         </is>
       </c>
       <c r="J290" t="inlineStr">
@@ -22689,7 +22689,7 @@
       </c>
       <c r="L290" t="inlineStr">
         <is>
-          <t>來孫子</t>
+          <t>來孫子 | 來孫</t>
         </is>
       </c>
       <c r="N290" t="inlineStr">
@@ -23136,7 +23136,7 @@
       </c>
       <c r="H296" t="inlineStr">
         <is>
-          <t>晜孫婿</t>
+          <t>晜孫婿 | 晜孫女婿</t>
         </is>
       </c>
       <c r="J296" t="inlineStr">
@@ -23151,7 +23151,7 @@
       </c>
       <c r="L296" t="inlineStr">
         <is>
-          <t>晜孫婿</t>
+          <t>晜孫婿 | 晜孫女婿</t>
         </is>
       </c>
       <c r="N296" t="inlineStr">
@@ -23213,7 +23213,7 @@
       </c>
       <c r="H297" t="inlineStr">
         <is>
-          <t>晜孫子</t>
+          <t>晜孫子 | 晜孫|昆孫</t>
         </is>
       </c>
       <c r="J297" t="inlineStr">
@@ -23228,7 +23228,7 @@
       </c>
       <c r="L297" t="inlineStr">
         <is>
-          <t>晜孫子</t>
+          <t>晜孫子 | 晜孫|昆孫</t>
         </is>
       </c>
       <c r="N297" t="inlineStr">
@@ -26678,7 +26678,7 @@
       </c>
       <c r="H342" t="inlineStr">
         <is>
-          <t>晜孫媳</t>
+          <t>晜孫媳 | 晜孫媳婦</t>
         </is>
       </c>
       <c r="J342" t="inlineStr">
@@ -26693,7 +26693,7 @@
       </c>
       <c r="L342" t="inlineStr">
         <is>
-          <t>晜孫媳</t>
+          <t>晜孫媳 | 晜孫媳婦</t>
         </is>
       </c>
       <c r="N342" t="inlineStr">
@@ -26755,7 +26755,7 @@
       </c>
       <c r="H343" t="inlineStr">
         <is>
-          <t>來孫媳</t>
+          <t>來孫媳 | 來孫媳婦</t>
         </is>
       </c>
       <c r="J343" t="inlineStr">
@@ -26770,7 +26770,7 @@
       </c>
       <c r="L343" t="inlineStr">
         <is>
-          <t>來孫媳</t>
+          <t>來孫媳 | 來孫媳婦</t>
         </is>
       </c>
       <c r="N343" t="inlineStr">
@@ -26832,7 +26832,7 @@
       </c>
       <c r="H344" t="inlineStr">
         <is>
-          <t>玄孫媳</t>
+          <t>玄孫媳 | 玄孫媳婦</t>
         </is>
       </c>
       <c r="J344" t="inlineStr">
@@ -26847,7 +26847,7 @@
       </c>
       <c r="L344" t="inlineStr">
         <is>
-          <t>玄孫媳</t>
+          <t>玄孫媳 | 玄孫媳婦</t>
         </is>
       </c>
       <c r="N344" t="inlineStr">
@@ -26909,7 +26909,7 @@
       </c>
       <c r="H345" t="inlineStr">
         <is>
-          <t>曾孫媳</t>
+          <t>曾孫媳 | 重孫媳婦|曾孫婦</t>
         </is>
       </c>
       <c r="J345" t="inlineStr">
@@ -26924,7 +26924,7 @@
       </c>
       <c r="L345" t="inlineStr">
         <is>
-          <t>曾孫媳</t>
+          <t>曾孫媳 | 重孫媳婦|曾孫婦</t>
         </is>
       </c>
       <c r="N345" t="inlineStr">
@@ -26986,7 +26986,7 @@
       </c>
       <c r="H346" t="inlineStr">
         <is>
-          <t>孫媳</t>
+          <t>孫媳 | 孫媳婦|孫新婦|孫婦</t>
         </is>
       </c>
       <c r="J346" t="inlineStr">
@@ -27001,7 +27001,7 @@
       </c>
       <c r="L346" t="inlineStr">
         <is>
-          <t>孫媳</t>
+          <t>孫媳 | 孫媳婦|孫新婦|孫婦</t>
         </is>
       </c>
       <c r="N346" t="inlineStr">
@@ -27063,7 +27063,7 @@
       </c>
       <c r="H347" t="inlineStr">
         <is>
-          <t>兒媳</t>
+          <t>兒媳 | 兒媳婦|兒媳婦兒|新婦|新婦囝|心抱|息婦|兒婦|子婦</t>
         </is>
       </c>
       <c r="J347" t="inlineStr">
@@ -27078,7 +27078,7 @@
       </c>
       <c r="L347" t="inlineStr">
         <is>
-          <t>兒媳</t>
+          <t>兒媳 | 兒媳婦|兒媳婦兒|新婦|新婦囝|心抱|息婦|兒婦|子婦</t>
         </is>
       </c>
       <c r="N347" t="inlineStr">
@@ -27371,7 +27371,7 @@
       </c>
       <c r="H351" t="inlineStr">
         <is>
-          <t>姻姪</t>
+          <t>姻姪 | 世姪</t>
         </is>
       </c>
       <c r="J351" t="inlineStr">
@@ -27386,7 +27386,7 @@
       </c>
       <c r="L351" t="inlineStr">
         <is>
-          <t>姻姪</t>
+          <t>姻姪 | 世姪</t>
         </is>
       </c>
       <c r="N351" t="inlineStr">
@@ -27987,7 +27987,7 @@
       </c>
       <c r="H359" t="inlineStr">
         <is>
-          <t>姻姪</t>
+          <t>姻姪 | 世姪</t>
         </is>
       </c>
       <c r="J359" t="inlineStr">
@@ -28002,7 +28002,7 @@
       </c>
       <c r="L359" t="inlineStr">
         <is>
-          <t>姻姪</t>
+          <t>姻姪 | 世姪</t>
         </is>
       </c>
       <c r="N359" t="inlineStr">
@@ -28603,22 +28603,22 @@
       </c>
       <c r="H367" t="inlineStr">
         <is>
+          <t>配偶 | 愛人|老伴|那口子|卿卿|老婆|太太|老太婆|老婆子|媳婦|媳婦兒|老婆兒|媳婦子|婆姨|婆娘|堂客|妻|娘子|夫人|內人|內子|內助|賢內助|愛妻|髮妻</t>
+        </is>
+      </c>
+      <c r="J367" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K367" t="inlineStr">
+        <is>
           <t>配偶</t>
         </is>
       </c>
-      <c r="J367" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="K367" t="inlineStr">
-        <is>
-          <t>配偶</t>
-        </is>
-      </c>
       <c r="L367" t="inlineStr">
         <is>
-          <t>配偶</t>
+          <t>配偶 | 愛人|老伴|那口子|卿卿|老公|先生|老頭子|漢子|夫|夫君|官人|郎君|相公|夫婿|良人</t>
         </is>
       </c>
       <c r="N367" t="inlineStr">
@@ -28680,7 +28680,7 @@
       </c>
       <c r="H368" t="inlineStr">
         <is>
-          <t>岳父 | 丈人|老丈人</t>
+          <t>岳父 | 丈人|老丈人|老公公|公爹|老親爺|丈人爹|老丈杆子|家公|大官|老人公|大人公|家官|丈人公|岳老子|外父|君舅|泰山|外舅|丈父|岳丈|岳翁|妻公|婦翁|冰翁</t>
         </is>
       </c>
       <c r="J368" t="inlineStr">
@@ -28757,7 +28757,7 @@
       </c>
       <c r="H369" t="inlineStr">
         <is>
-          <t>岳祖父</t>
+          <t>岳祖父 | 祖公公|祖岳父|太岳父</t>
         </is>
       </c>
       <c r="J369" t="inlineStr">
@@ -28772,7 +28772,7 @@
       </c>
       <c r="L369" t="inlineStr">
         <is>
-          <t>祖父</t>
+          <t>祖父 | 爺爺|爺|阿公|祖公|阿爺|依爺|嗲嗲|亞爺|亞公|大父|祖翁</t>
         </is>
       </c>
       <c r="N369" t="inlineStr">
@@ -28849,7 +28849,7 @@
       </c>
       <c r="L370" t="inlineStr">
         <is>
-          <t>曾祖父</t>
+          <t>曾祖父 | 太爺爺|太爺|老太爺|曾爺爺|太公|佬嗲|公太|曾祖|太翁</t>
         </is>
       </c>
       <c r="N370" t="inlineStr">
@@ -28926,7 +28926,7 @@
       </c>
       <c r="L371" t="inlineStr">
         <is>
-          <t>伯曾祖父</t>
+          <t>伯曾祖父 | 太公</t>
         </is>
       </c>
       <c r="N371" t="inlineStr">
@@ -29003,7 +29003,7 @@
       </c>
       <c r="L372" t="inlineStr">
         <is>
-          <t>伯曾祖母</t>
+          <t>伯曾祖母 | 太婆</t>
         </is>
       </c>
       <c r="N372" t="inlineStr">
@@ -29080,7 +29080,7 @@
       </c>
       <c r="L373" t="inlineStr">
         <is>
-          <t>姑曾祖母</t>
+          <t>姑曾祖母 | 太婆</t>
         </is>
       </c>
       <c r="N373" t="inlineStr">
@@ -29234,7 +29234,7 @@
       </c>
       <c r="L375" t="inlineStr">
         <is>
-          <t>叔曾祖父</t>
+          <t>叔曾祖父 | 太公</t>
         </is>
       </c>
       <c r="N375" t="inlineStr">
@@ -29311,7 +29311,7 @@
       </c>
       <c r="L376" t="inlineStr">
         <is>
-          <t>叔曾祖母</t>
+          <t>叔曾祖母 | 太婆</t>
         </is>
       </c>
       <c r="N376" t="inlineStr">
@@ -29388,7 +29388,7 @@
       </c>
       <c r="L377" t="inlineStr">
         <is>
-          <t>姑曾祖母</t>
+          <t>姑曾祖母 | 太婆</t>
         </is>
       </c>
       <c r="N377" t="inlineStr">
@@ -29542,7 +29542,7 @@
       </c>
       <c r="L379" t="inlineStr">
         <is>
-          <t>曾祖母</t>
+          <t>曾祖母 | 太奶奶|太奶|老太奶|曾奶奶|太婆|太嬤|太姆|老娭毑|婆太</t>
         </is>
       </c>
       <c r="N379" t="inlineStr">
@@ -29619,7 +29619,7 @@
       </c>
       <c r="L380" t="inlineStr">
         <is>
-          <t>堂伯</t>
+          <t>堂伯 | 從父</t>
         </is>
       </c>
       <c r="N380" t="inlineStr">
@@ -29773,7 +29773,7 @@
       </c>
       <c r="L382" t="inlineStr">
         <is>
-          <t>堂叔</t>
+          <t>堂叔 | 從父</t>
         </is>
       </c>
       <c r="N382" t="inlineStr">
@@ -29912,7 +29912,7 @@
       </c>
       <c r="H384" t="inlineStr">
         <is>
-          <t>岳祖母</t>
+          <t>岳祖母 | 祖丈母|祖丈母娘|祖婆婆|祖岳母|太岳母</t>
         </is>
       </c>
       <c r="J384" t="inlineStr">
@@ -29927,7 +29927,7 @@
       </c>
       <c r="L384" t="inlineStr">
         <is>
-          <t>祖母</t>
+          <t>祖母 | 奶奶|奶|阿嬤|祖嫲|祖婆|依奶|阿奶|阿婆|親婆|娭毑|亞嬤|亞婆|嫲嫲|大母</t>
         </is>
       </c>
       <c r="N384" t="inlineStr">
@@ -30004,7 +30004,7 @@
       </c>
       <c r="L385" t="inlineStr">
         <is>
-          <t>曾外祖父</t>
+          <t>曾外祖父 | 太外爺|太外爺爺|太外公|曾外祖</t>
         </is>
       </c>
       <c r="N385" t="inlineStr">
@@ -30081,7 +30081,7 @@
       </c>
       <c r="L386" t="inlineStr">
         <is>
-          <t>曾外祖母</t>
+          <t>曾外祖母 | 太外奶|太外奶奶|太外婆</t>
         </is>
       </c>
       <c r="N386" t="inlineStr">
@@ -30143,7 +30143,7 @@
       </c>
       <c r="H387" t="inlineStr">
         <is>
-          <t>伯岳父 | 伯公</t>
+          <t>伯岳父 | 伯公|伯公公</t>
         </is>
       </c>
       <c r="J387" t="inlineStr">
@@ -30158,7 +30158,7 @@
       </c>
       <c r="L387" t="inlineStr">
         <is>
-          <t>伯岳父 | 伯公</t>
+          <t>伯岳父 | 伯公|伯公公</t>
         </is>
       </c>
       <c r="N387" t="inlineStr">
@@ -30215,32 +30215,32 @@
       </c>
       <c r="G388" t="inlineStr">
         <is>
-          <t>配偶的父的兄的配偶</t>
+          <t>配偶的旁係長輩</t>
         </is>
       </c>
       <c r="H388" t="inlineStr">
         <is>
-          <t>配偶的父的兄的配偶</t>
+          <t>伯岳母 | 伯婆</t>
         </is>
       </c>
       <c r="J388" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="K388" t="inlineStr">
         <is>
-          <t>配偶的父的兄的配偶</t>
+          <t>配偶的旁係長輩</t>
         </is>
       </c>
       <c r="L388" t="inlineStr">
         <is>
-          <t>配偶的父的兄的配偶</t>
+          <t>伯岳母 | 伯婆</t>
         </is>
       </c>
       <c r="N388" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="O388" t="inlineStr">
@@ -30250,12 +30250,12 @@
       </c>
       <c r="P388" t="inlineStr">
         <is>
-          <t>配偶的父的兄的配偶</t>
+          <t>伯岳母</t>
         </is>
       </c>
       <c r="Q388" t="inlineStr">
         <is>
-          <t>已收編：配偶的父的兄的配偶</t>
+          <t>一致</t>
         </is>
       </c>
     </row>
@@ -30369,32 +30369,32 @@
       </c>
       <c r="G390" t="inlineStr">
         <is>
-          <t>配偶的父的姐的配偶</t>
+          <t>配偶的旁係長輩</t>
         </is>
       </c>
       <c r="H390" t="inlineStr">
         <is>
-          <t>配偶的父的姐的配偶</t>
+          <t>姑岳父 | 姑公</t>
         </is>
       </c>
       <c r="J390" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="K390" t="inlineStr">
         <is>
-          <t>配偶的父的姐的配偶</t>
+          <t>配偶的旁係長輩</t>
         </is>
       </c>
       <c r="L390" t="inlineStr">
         <is>
-          <t>配偶的父的姐的配偶</t>
+          <t>姑岳父 | 姑公</t>
         </is>
       </c>
       <c r="N390" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="O390" t="inlineStr">
@@ -30404,12 +30404,12 @@
       </c>
       <c r="P390" t="inlineStr">
         <is>
-          <t>配偶的父的姐的配偶</t>
+          <t>姑岳父（候選命中：姑公）</t>
         </is>
       </c>
       <c r="Q390" t="inlineStr">
         <is>
-          <t>已收編：配偶的父的姐的配偶</t>
+          <t>可接受簡寫：姑岳父（候選命中：姑公）</t>
         </is>
       </c>
     </row>
@@ -30451,7 +30451,7 @@
       </c>
       <c r="H391" t="inlineStr">
         <is>
-          <t>叔岳父 | 叔公</t>
+          <t>叔岳父 | 叔公|叔公公</t>
         </is>
       </c>
       <c r="J391" t="inlineStr">
@@ -30466,7 +30466,7 @@
       </c>
       <c r="L391" t="inlineStr">
         <is>
-          <t>叔岳父 | 叔公</t>
+          <t>叔岳父 | 叔公|叔公公</t>
         </is>
       </c>
       <c r="N391" t="inlineStr">
@@ -30523,32 +30523,32 @@
       </c>
       <c r="G392" t="inlineStr">
         <is>
-          <t>配偶的父的弟的配偶</t>
+          <t>配偶的旁係長輩</t>
         </is>
       </c>
       <c r="H392" t="inlineStr">
         <is>
-          <t>配偶的父的弟的配偶</t>
+          <t>叔岳母 | 叔婆</t>
         </is>
       </c>
       <c r="J392" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="K392" t="inlineStr">
         <is>
-          <t>配偶的父的弟的配偶</t>
+          <t>配偶的旁係長輩</t>
         </is>
       </c>
       <c r="L392" t="inlineStr">
         <is>
-          <t>配偶的父的弟的配偶</t>
+          <t>叔岳母 | 叔婆</t>
         </is>
       </c>
       <c r="N392" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="O392" t="inlineStr">
@@ -30558,12 +30558,12 @@
       </c>
       <c r="P392" t="inlineStr">
         <is>
-          <t>配偶的父的弟的配偶</t>
+          <t>叔岳母</t>
         </is>
       </c>
       <c r="Q392" t="inlineStr">
         <is>
-          <t>已收編：配偶的父的弟的配偶</t>
+          <t>一致</t>
         </is>
       </c>
     </row>
@@ -30677,32 +30677,32 @@
       </c>
       <c r="G394" t="inlineStr">
         <is>
-          <t>配偶的父的妹的配偶</t>
+          <t>配偶的旁係長輩</t>
         </is>
       </c>
       <c r="H394" t="inlineStr">
         <is>
-          <t>配偶的父的妹的配偶</t>
+          <t>姑岳父 | 姑公</t>
         </is>
       </c>
       <c r="J394" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="K394" t="inlineStr">
         <is>
-          <t>配偶的父的妹的配偶</t>
+          <t>配偶的旁係長輩</t>
         </is>
       </c>
       <c r="L394" t="inlineStr">
         <is>
-          <t>配偶的父的妹的配偶</t>
+          <t>姑岳父 | 姑公</t>
         </is>
       </c>
       <c r="N394" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="O394" t="inlineStr">
@@ -30712,12 +30712,12 @@
       </c>
       <c r="P394" t="inlineStr">
         <is>
-          <t>配偶的父的妹的配偶</t>
+          <t>姑岳父（候選命中：姑公）</t>
         </is>
       </c>
       <c r="Q394" t="inlineStr">
         <is>
-          <t>已收編：配偶的父的妹的配偶</t>
+          <t>可接受簡寫：姑岳父（候選命中：姑公）</t>
         </is>
       </c>
     </row>
@@ -30759,7 +30759,7 @@
       </c>
       <c r="H395" t="inlineStr">
         <is>
-          <t>岳母 | 丈母娘</t>
+          <t>岳母 | 丈母|丈母娘|婆母|老婆婆|老丈母|老親娘|家婆|家娘|老人婆|大人婆|阿姑|婆母娘|岳母娘|丈母婆|丈人娘|丈人婆|丈姆|丈姆婆|丈姆娘|外母|大家|君姑|泰水|外姑</t>
         </is>
       </c>
       <c r="J395" t="inlineStr">
@@ -30836,7 +30836,7 @@
       </c>
       <c r="H396" t="inlineStr">
         <is>
-          <t>岳外祖父</t>
+          <t>岳外祖父 | 姥丈人|外祖公</t>
         </is>
       </c>
       <c r="J396" t="inlineStr">
@@ -30851,7 +30851,7 @@
       </c>
       <c r="L396" t="inlineStr">
         <is>
-          <t>外祖父</t>
+          <t>外祖父 | 姥爺|姥公|舅家爺|姥爹|外公|外爺|尕公|嘎公|嘎爹|嘎嘎爹|嘎爺爺|毑父|毑公|毑爹|毑爺|外大父</t>
         </is>
       </c>
       <c r="N396" t="inlineStr">
@@ -30928,7 +30928,7 @@
       </c>
       <c r="L397" t="inlineStr">
         <is>
-          <t>外曾祖父</t>
+          <t>外曾祖父 | 外太爺爺|外太爺|外太公|外曾祖</t>
         </is>
       </c>
       <c r="N397" t="inlineStr">
@@ -31005,7 +31005,7 @@
       </c>
       <c r="L398" t="inlineStr">
         <is>
-          <t>外曾祖母</t>
+          <t>外曾祖母 | 外太奶奶|外太奶|外太婆</t>
         </is>
       </c>
       <c r="N398" t="inlineStr">
@@ -31067,7 +31067,7 @@
       </c>
       <c r="H399" t="inlineStr">
         <is>
-          <t>岳外祖母</t>
+          <t>岳外祖母 | 姥丈母|外祖婆</t>
         </is>
       </c>
       <c r="J399" t="inlineStr">
@@ -31082,7 +31082,7 @@
       </c>
       <c r="L399" t="inlineStr">
         <is>
-          <t>外祖母</t>
+          <t>外祖母 | 姥姥|外奶|姥婆|舅家婆|姥娘|姥|外婆|外嬤|尕婆|嘎嘎|嘎婆|嘎嘎婆|嘎奶奶|阿婆|好婆|毑母|毑婆|毑娘|毑毑|嫲嫲|外大母</t>
         </is>
       </c>
       <c r="N399" t="inlineStr">
@@ -31159,7 +31159,7 @@
       </c>
       <c r="L400" t="inlineStr">
         <is>
-          <t>外曾外祖父</t>
+          <t>外曾外祖父 | 外太姥爺|曾毑父|外曾外祖</t>
         </is>
       </c>
       <c r="N400" t="inlineStr">
@@ -31236,7 +31236,7 @@
       </c>
       <c r="L401" t="inlineStr">
         <is>
-          <t>外曾外祖母</t>
+          <t>外曾外祖母 | 外太姥姥|曾毑母</t>
         </is>
       </c>
       <c r="N401" t="inlineStr">
@@ -31370,32 +31370,32 @@
       </c>
       <c r="G403" t="inlineStr">
         <is>
-          <t>配偶的母的兄的配偶</t>
+          <t>配偶的旁係長輩</t>
         </is>
       </c>
       <c r="H403" t="inlineStr">
         <is>
-          <t>配偶的母的兄的配偶</t>
+          <t>舅岳母 | 舅婆</t>
         </is>
       </c>
       <c r="J403" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="K403" t="inlineStr">
         <is>
-          <t>配偶的母的兄的配偶</t>
+          <t>配偶的旁係長輩</t>
         </is>
       </c>
       <c r="L403" t="inlineStr">
         <is>
-          <t>配偶的母的兄的配偶</t>
+          <t>舅岳母 | 舅婆</t>
         </is>
       </c>
       <c r="N403" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="O403" t="inlineStr">
@@ -31405,12 +31405,12 @@
       </c>
       <c r="P403" t="inlineStr">
         <is>
-          <t>配偶的母的兄的配偶</t>
+          <t>舅岳母（候選命中：舅婆）</t>
         </is>
       </c>
       <c r="Q403" t="inlineStr">
         <is>
-          <t>已收編：配偶的母的兄的配偶</t>
+          <t>可接受簡寫：舅岳母（候選命中：舅婆）</t>
         </is>
       </c>
     </row>
@@ -31524,32 +31524,32 @@
       </c>
       <c r="G405" t="inlineStr">
         <is>
-          <t>配偶的母的姐的配偶</t>
+          <t>配偶的旁係長輩</t>
         </is>
       </c>
       <c r="H405" t="inlineStr">
         <is>
-          <t>配偶的母的姐的配偶</t>
+          <t>姨岳父 | 姨公</t>
         </is>
       </c>
       <c r="J405" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="K405" t="inlineStr">
         <is>
-          <t>配偶的母的姐的配偶</t>
+          <t>配偶的旁係長輩</t>
         </is>
       </c>
       <c r="L405" t="inlineStr">
         <is>
-          <t>配偶的母的姐的配偶</t>
+          <t>姨岳父 | 姨公</t>
         </is>
       </c>
       <c r="N405" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="O405" t="inlineStr">
@@ -31559,12 +31559,12 @@
       </c>
       <c r="P405" t="inlineStr">
         <is>
-          <t>配偶的母的姐的配偶</t>
+          <t>姨岳父（候選命中：姨公）</t>
         </is>
       </c>
       <c r="Q405" t="inlineStr">
         <is>
-          <t>已收編：配偶的母的姐的配偶</t>
+          <t>可接受簡寫：姨岳父（候選命中：姨公）</t>
         </is>
       </c>
     </row>
@@ -31678,32 +31678,32 @@
       </c>
       <c r="G407" t="inlineStr">
         <is>
-          <t>配偶的母的弟的配偶</t>
+          <t>配偶的旁係長輩</t>
         </is>
       </c>
       <c r="H407" t="inlineStr">
         <is>
-          <t>配偶的母的弟的配偶</t>
+          <t>舅岳母 | 舅婆</t>
         </is>
       </c>
       <c r="J407" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="K407" t="inlineStr">
         <is>
-          <t>配偶的母的弟的配偶</t>
+          <t>配偶的旁係長輩</t>
         </is>
       </c>
       <c r="L407" t="inlineStr">
         <is>
-          <t>配偶的母的弟的配偶</t>
+          <t>舅岳母 | 舅婆</t>
         </is>
       </c>
       <c r="N407" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="O407" t="inlineStr">
@@ -31713,12 +31713,12 @@
       </c>
       <c r="P407" t="inlineStr">
         <is>
-          <t>配偶的母的弟的配偶</t>
+          <t>舅岳母（候選命中：舅婆）</t>
         </is>
       </c>
       <c r="Q407" t="inlineStr">
         <is>
-          <t>已收編：配偶的母的弟的配偶</t>
+          <t>可接受簡寫：舅岳母（候選命中：舅婆）</t>
         </is>
       </c>
     </row>
@@ -31832,32 +31832,32 @@
       </c>
       <c r="G409" t="inlineStr">
         <is>
-          <t>配偶的母的妹的配偶</t>
+          <t>配偶的旁係長輩</t>
         </is>
       </c>
       <c r="H409" t="inlineStr">
         <is>
-          <t>配偶的母的妹的配偶</t>
+          <t>姨岳父 | 姨公</t>
         </is>
       </c>
       <c r="J409" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="K409" t="inlineStr">
         <is>
-          <t>配偶的母的妹的配偶</t>
+          <t>配偶的旁係長輩</t>
         </is>
       </c>
       <c r="L409" t="inlineStr">
         <is>
-          <t>配偶的母的妹的配偶</t>
+          <t>姨岳父 | 姨公</t>
         </is>
       </c>
       <c r="N409" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="O409" t="inlineStr">
@@ -31867,12 +31867,12 @@
       </c>
       <c r="P409" t="inlineStr">
         <is>
-          <t>配偶的母的妹的配偶</t>
+          <t>姨岳父（候選命中：姨公）</t>
         </is>
       </c>
       <c r="Q409" t="inlineStr">
         <is>
-          <t>已收編：配偶的母的妹的配偶</t>
+          <t>可接受簡寫：姨岳父（候選命中：姨公）</t>
         </is>
       </c>
     </row>
@@ -31914,7 +31914,7 @@
       </c>
       <c r="H410" t="inlineStr">
         <is>
-          <t>大舅子 | 大舅哥</t>
+          <t>大舅子 | 大舅哥|舅子|大阿舅|舅哥|丈人兄|妻舅</t>
         </is>
       </c>
       <c r="J410" t="inlineStr">
@@ -31991,7 +31991,7 @@
       </c>
       <c r="H411" t="inlineStr">
         <is>
-          <t>內姪女</t>
+          <t>內姪女 | 舅姪女</t>
         </is>
       </c>
       <c r="J411" t="inlineStr">
@@ -32006,7 +32006,7 @@
       </c>
       <c r="L411" t="inlineStr">
         <is>
-          <t>姪女</t>
+          <t>姪女 | 姪女兒|姪丫頭|姪閨女|姪囡|兄女</t>
         </is>
       </c>
       <c r="N411" t="inlineStr">
@@ -32021,12 +32021,12 @@
       </c>
       <c r="P411" t="inlineStr">
         <is>
-          <t>男：內姪女；女：姪女</t>
+          <t>男：內姪女；女：姪女（候選命中：舅侄女）</t>
         </is>
       </c>
       <c r="Q411" t="inlineStr">
         <is>
-          <t>已收編：男：內姪女；女：姪女</t>
+          <t>已收編：男：內姪女；女：姪女（候選命中：舅侄女）</t>
         </is>
       </c>
     </row>
@@ -32068,7 +32068,7 @@
       </c>
       <c r="H412" t="inlineStr">
         <is>
-          <t>內姪</t>
+          <t>內姪 | 舅姪</t>
         </is>
       </c>
       <c r="J412" t="inlineStr">
@@ -32098,12 +32098,12 @@
       </c>
       <c r="P412" t="inlineStr">
         <is>
-          <t>男：內姪；女：姪</t>
+          <t>男：內姪；女：姪（候選命中：舅侄）</t>
         </is>
       </c>
       <c r="Q412" t="inlineStr">
         <is>
-          <t>已收編：男：內姪；女：姪</t>
+          <t>已收編：男：內姪；女：姪（候選命中：舅侄）</t>
         </is>
       </c>
     </row>
@@ -32145,7 +32145,7 @@
       </c>
       <c r="H413" t="inlineStr">
         <is>
-          <t>舅嫂 | 大舅嫂</t>
+          <t>舅嫂 | 大舅嫂|大妗子|大妗兒|妻妗</t>
         </is>
       </c>
       <c r="J413" t="inlineStr">
@@ -32222,7 +32222,7 @@
       </c>
       <c r="H414" t="inlineStr">
         <is>
-          <t>大姨子 | 大姨姐</t>
+          <t>大姨子 | 大姨姐|姨姐|大姨兒</t>
         </is>
       </c>
       <c r="J414" t="inlineStr">
@@ -32453,7 +32453,7 @@
       </c>
       <c r="H417" t="inlineStr">
         <is>
-          <t>姐夫 | 連襟</t>
+          <t>襟兄 | 連襟|姐夫|老襟|一擔挑|老挑|挑擔|擔兒挑|連襟兒|連橋|兩橋|友婿|婭</t>
         </is>
       </c>
       <c r="J417" t="inlineStr">
@@ -32468,7 +32468,7 @@
       </c>
       <c r="L417" t="inlineStr">
         <is>
-          <t>姐夫</t>
+          <t>姐夫 | 姐丈|姐夫哥|姐婿</t>
         </is>
       </c>
       <c r="N417" t="inlineStr">
@@ -32483,12 +32483,12 @@
       </c>
       <c r="P417" t="inlineStr">
         <is>
-          <t>姐夫</t>
+          <t>男：襟兄；女：姐夫</t>
         </is>
       </c>
       <c r="Q417" t="inlineStr">
         <is>
-          <t>已收編：姐夫</t>
+          <t>已收編：男：襟兄；女：姐夫</t>
         </is>
       </c>
     </row>
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H418" t="inlineStr">
         <is>
-          <t>小舅子</t>
+          <t>小舅子 | 小舅弟|舅弟|小阿舅|丈人弟</t>
         </is>
       </c>
       <c r="J418" t="inlineStr">
@@ -32607,7 +32607,7 @@
       </c>
       <c r="H419" t="inlineStr">
         <is>
-          <t>內姪女</t>
+          <t>內姪女 | 舅姪女</t>
         </is>
       </c>
       <c r="J419" t="inlineStr">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="L419" t="inlineStr">
         <is>
-          <t>姪女</t>
+          <t>姪女 | 姪女兒|姪丫頭|姪閨女|姪囡|兄女</t>
         </is>
       </c>
       <c r="N419" t="inlineStr">
@@ -32637,12 +32637,12 @@
       </c>
       <c r="P419" t="inlineStr">
         <is>
-          <t>男：內姪女；女：姪女</t>
+          <t>男：內姪女；女：姪女（候選命中：舅侄女）</t>
         </is>
       </c>
       <c r="Q419" t="inlineStr">
         <is>
-          <t>已收編：男：內姪女；女：姪女</t>
+          <t>已收編：男：內姪女；女：姪女（候選命中：舅侄女）</t>
         </is>
       </c>
     </row>
@@ -32684,7 +32684,7 @@
       </c>
       <c r="H420" t="inlineStr">
         <is>
-          <t>內姪</t>
+          <t>內姪 | 舅姪</t>
         </is>
       </c>
       <c r="J420" t="inlineStr">
@@ -32714,12 +32714,12 @@
       </c>
       <c r="P420" t="inlineStr">
         <is>
-          <t>男：內姪；女：姪</t>
+          <t>男：內姪；女：姪（候選命中：舅侄）</t>
         </is>
       </c>
       <c r="Q420" t="inlineStr">
         <is>
-          <t>已收編：男：內姪；女：姪</t>
+          <t>已收編：男：內姪；女：姪（候選命中：舅侄）</t>
         </is>
       </c>
     </row>
@@ -32761,7 +32761,7 @@
       </c>
       <c r="H421" t="inlineStr">
         <is>
-          <t>弟妹 | 舅弟媳</t>
+          <t>弟妹 | 舅弟媳|小妗子|小妗兒</t>
         </is>
       </c>
       <c r="J421" t="inlineStr">
@@ -32776,7 +32776,7 @@
       </c>
       <c r="L421" t="inlineStr">
         <is>
-          <t>弟妹 | 弟媳</t>
+          <t>弟妹 | 弟媳|小妗子|小妗兒</t>
         </is>
       </c>
       <c r="N421" t="inlineStr">
@@ -32796,7 +32796,7 @@
       </c>
       <c r="Q421" t="inlineStr">
         <is>
-          <t>已收編：弟妹（候選命中：舅弟媳）</t>
+          <t>可接受簡寫：弟妹（候選命中：舅弟媳）</t>
         </is>
       </c>
     </row>
@@ -32838,7 +32838,7 @@
       </c>
       <c r="H422" t="inlineStr">
         <is>
-          <t>小姨子 | 小姨妹</t>
+          <t>小姨子 | 小姨妹|姨子|姨妹|姨妹子|妻姨</t>
         </is>
       </c>
       <c r="J422" t="inlineStr">
@@ -33069,7 +33069,7 @@
       </c>
       <c r="H425" t="inlineStr">
         <is>
-          <t>妹夫 | 連襟</t>
+          <t>襟弟 | 連襟|妹夫|老襟|一擔挑|老挑|挑擔|擔兒挑|連襟兒|連橋|兩橋|友婿|婭</t>
         </is>
       </c>
       <c r="J425" t="inlineStr">
@@ -33084,7 +33084,7 @@
       </c>
       <c r="L425" t="inlineStr">
         <is>
-          <t>妹夫</t>
+          <t>妹夫 | 妹丈|妹婿</t>
         </is>
       </c>
       <c r="N425" t="inlineStr">
@@ -33099,12 +33099,12 @@
       </c>
       <c r="P425" t="inlineStr">
         <is>
-          <t>妹夫</t>
+          <t>男：襟弟；女：妹夫</t>
         </is>
       </c>
       <c r="Q425" t="inlineStr">
         <is>
-          <t>已收編：妹夫</t>
+          <t>已收編：男：襟弟；女：妹夫</t>
         </is>
       </c>
     </row>
@@ -33146,22 +33146,22 @@
       </c>
       <c r="H426" t="inlineStr">
         <is>
+          <t>弟弟 | 弟|親弟|老弟|小弟|依弟|阿弟|細佬|胞弟</t>
+        </is>
+      </c>
+      <c r="J426" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K426" t="inlineStr">
+        <is>
           <t>弟弟</t>
         </is>
       </c>
-      <c r="J426" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="K426" t="inlineStr">
-        <is>
-          <t>弟弟</t>
-        </is>
-      </c>
       <c r="L426" t="inlineStr">
         <is>
-          <t>弟弟</t>
+          <t>弟弟 | 弟|親弟|老弟|小弟|依弟|阿弟|細佬|胞弟</t>
         </is>
       </c>
       <c r="N426" t="inlineStr">
@@ -33223,7 +33223,7 @@
       </c>
       <c r="H427" t="inlineStr">
         <is>
-          <t>姪女</t>
+          <t>姪女 | 姪女兒|姪丫頭|姪閨女|姪囡|兄女</t>
         </is>
       </c>
       <c r="J427" t="inlineStr">
@@ -33238,7 +33238,7 @@
       </c>
       <c r="L427" t="inlineStr">
         <is>
-          <t>姪女</t>
+          <t>姪女 | 姪女兒|姪丫頭|姪閨女|姪囡|兄女</t>
         </is>
       </c>
       <c r="N427" t="inlineStr">
@@ -33300,7 +33300,7 @@
       </c>
       <c r="H428" t="inlineStr">
         <is>
-          <t>姪女婿</t>
+          <t>姪女婿 | 姪婿</t>
         </is>
       </c>
       <c r="J428" t="inlineStr">
@@ -33315,7 +33315,7 @@
       </c>
       <c r="L428" t="inlineStr">
         <is>
-          <t>姪女婿</t>
+          <t>姪女婿 | 姪婿</t>
         </is>
       </c>
       <c r="N428" t="inlineStr">
@@ -33377,7 +33377,7 @@
       </c>
       <c r="H429" t="inlineStr">
         <is>
-          <t>姪子</t>
+          <t>姪子 | 親姪|姪兒|姪|姪小子|老姪|姪仔|阿姪|兄子|姪男|嫡姪</t>
         </is>
       </c>
       <c r="J429" t="inlineStr">
@@ -33392,7 +33392,7 @@
       </c>
       <c r="L429" t="inlineStr">
         <is>
-          <t>姪子</t>
+          <t>姪子 | 親姪|姪兒|姪|姪小子|老姪|姪仔|阿姪|兄子|姪男|嫡姪</t>
         </is>
       </c>
       <c r="N429" t="inlineStr">
@@ -33454,7 +33454,7 @@
       </c>
       <c r="H430" t="inlineStr">
         <is>
-          <t>姪媳婦</t>
+          <t>姪媳婦 | 姪媳|姪婦</t>
         </is>
       </c>
       <c r="J430" t="inlineStr">
@@ -33469,7 +33469,7 @@
       </c>
       <c r="L430" t="inlineStr">
         <is>
-          <t>姪媳婦</t>
+          <t>姪媳婦 | 姪媳|姪婦</t>
         </is>
       </c>
       <c r="N430" t="inlineStr">
@@ -33531,7 +33531,7 @@
       </c>
       <c r="H431" t="inlineStr">
         <is>
-          <t>弟媳 | 弟妹</t>
+          <t>弟媳 | 弟妹|弟媳婦|弟新婦|弟媳婦子</t>
         </is>
       </c>
       <c r="J431" t="inlineStr">
@@ -33546,7 +33546,7 @@
       </c>
       <c r="L431" t="inlineStr">
         <is>
-          <t>弟媳 | 弟妹</t>
+          <t>弟媳 | 弟妹|弟媳婦|弟新婦|弟媳婦子</t>
         </is>
       </c>
       <c r="N431" t="inlineStr">
@@ -33608,22 +33608,22 @@
       </c>
       <c r="H432" t="inlineStr">
         <is>
+          <t>妹妹 | 妹|親妹|老妹|小妹|阿妹|依妹|妹子|妹兒|胞妹</t>
+        </is>
+      </c>
+      <c r="J432" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K432" t="inlineStr">
+        <is>
           <t>妹妹</t>
         </is>
       </c>
-      <c r="J432" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="K432" t="inlineStr">
-        <is>
-          <t>妹妹</t>
-        </is>
-      </c>
       <c r="L432" t="inlineStr">
         <is>
-          <t>妹妹</t>
+          <t>妹妹 | 妹|親妹|老妹|小妹|阿妹|依妹|妹子|妹兒|胞妹</t>
         </is>
       </c>
       <c r="N432" t="inlineStr">
@@ -33685,7 +33685,7 @@
       </c>
       <c r="H433" t="inlineStr">
         <is>
-          <t>外甥女</t>
+          <t>外甥女 | 甥女兒|甥閨女|甥囡|甥女</t>
         </is>
       </c>
       <c r="J433" t="inlineStr">
@@ -33700,7 +33700,7 @@
       </c>
       <c r="L433" t="inlineStr">
         <is>
-          <t>外甥女</t>
+          <t>外甥女 | 甥女兒|甥閨女|甥囡|甥女</t>
         </is>
       </c>
       <c r="N433" t="inlineStr">
@@ -33762,7 +33762,7 @@
       </c>
       <c r="H434" t="inlineStr">
         <is>
-          <t>外甥婿</t>
+          <t>外甥婿 | 甥女婿|甥婿</t>
         </is>
       </c>
       <c r="J434" t="inlineStr">
@@ -33777,7 +33777,7 @@
       </c>
       <c r="L434" t="inlineStr">
         <is>
-          <t>外甥婿</t>
+          <t>外甥婿 | 甥女婿|甥婿</t>
         </is>
       </c>
       <c r="N434" t="inlineStr">
@@ -33839,7 +33839,7 @@
       </c>
       <c r="H435" t="inlineStr">
         <is>
-          <t>外甥</t>
+          <t>外甥 | 甥兒|甥仔|甥子|甥男|甥</t>
         </is>
       </c>
       <c r="J435" t="inlineStr">
@@ -33854,7 +33854,7 @@
       </c>
       <c r="L435" t="inlineStr">
         <is>
-          <t>外甥</t>
+          <t>外甥 | 甥兒|甥仔|甥子|甥男|甥</t>
         </is>
       </c>
       <c r="N435" t="inlineStr">
@@ -33916,7 +33916,7 @@
       </c>
       <c r="H436" t="inlineStr">
         <is>
-          <t>外甥孫女</t>
+          <t>外甥孫女 | 甥孫女|遠甥女|彌甥女</t>
         </is>
       </c>
       <c r="J436" t="inlineStr">
@@ -33931,7 +33931,7 @@
       </c>
       <c r="L436" t="inlineStr">
         <is>
-          <t>外甥孫女</t>
+          <t>外甥孫女 | 甥孫女|遠甥女|彌甥女</t>
         </is>
       </c>
       <c r="N436" t="inlineStr">
@@ -33993,7 +33993,7 @@
       </c>
       <c r="H437" t="inlineStr">
         <is>
-          <t>外甥孫</t>
+          <t>外甥孫 | 甥孫|遠甥|彌甥</t>
         </is>
       </c>
       <c r="J437" t="inlineStr">
@@ -34008,7 +34008,7 @@
       </c>
       <c r="L437" t="inlineStr">
         <is>
-          <t>外甥孫</t>
+          <t>外甥孫 | 甥孫|遠甥|彌甥</t>
         </is>
       </c>
       <c r="N437" t="inlineStr">
@@ -34070,7 +34070,7 @@
       </c>
       <c r="H438" t="inlineStr">
         <is>
-          <t>外甥媳</t>
+          <t>外甥媳 | 甥媳婦|甥媳|甥婦</t>
         </is>
       </c>
       <c r="J438" t="inlineStr">
@@ -34085,7 +34085,7 @@
       </c>
       <c r="L438" t="inlineStr">
         <is>
-          <t>外甥媳</t>
+          <t>外甥媳 | 甥媳婦|甥媳|甥婦</t>
         </is>
       </c>
       <c r="N438" t="inlineStr">
@@ -34147,7 +34147,7 @@
       </c>
       <c r="H439" t="inlineStr">
         <is>
-          <t>妹夫 | 連襟</t>
+          <t>妹夫 | 妹丈|妹婿</t>
         </is>
       </c>
       <c r="J439" t="inlineStr">
@@ -34162,7 +34162,7 @@
       </c>
       <c r="L439" t="inlineStr">
         <is>
-          <t>妹夫 | 連襟</t>
+          <t>妹夫 | 妹丈|妹婿</t>
         </is>
       </c>
       <c r="N439" t="inlineStr">

</xml_diff>